<commit_message>
Updated report with NMDS, PERMANOVA, and RDA.
</commit_message>
<xml_diff>
--- a/2025greenhouse/2025greenhousemaster.xlsx
+++ b/2025greenhouse/2025greenhousemaster.xlsx
@@ -1,20 +1,27 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10208"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10215"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/reneedavis/R/Biobead/2025greenhouse/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B00D2D79-A656-924C-B36A-6BD8B90636AF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E0E29788-C20D-EE44-9942-A5A86D2D3A31}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="1380" yWindow="1060" windowWidth="25260" windowHeight="15800" xr2:uid="{F83686B1-B1F8-0E46-8563-14D114C6B912}"/>
+    <workbookView xWindow="1060" yWindow="920" windowWidth="25260" windowHeight="15800" xr2:uid="{F83686B1-B1F8-0E46-8563-14D114C6B912}"/>
   </bookViews>
   <sheets>
     <sheet name="Master" sheetId="1" r:id="rId1"/>
   </sheets>
+  <definedNames>
+    <definedName name="_xlchart.v1.0" hidden="1">Master!$C$2:$C$99</definedName>
+    <definedName name="_xlchart.v1.1" hidden="1">Master!$H$2:$H$99</definedName>
+    <definedName name="_xlchart.v1.2" hidden="1">Master!$H$2:$H$99</definedName>
+    <definedName name="_xlchart.v1.3" hidden="1">Master!$F$2:$F$99</definedName>
+    <definedName name="_xlchart.v1.4" hidden="1">Master!$F$2:$F$99</definedName>
+  </definedNames>
   <calcPr calcId="191029"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
@@ -443,11 +450,9 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="5">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
@@ -794,7 +799,7 @@
     <col min="9" max="16384" width="10.83203125" style="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:24" s="1" customFormat="1" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:24" x14ac:dyDescent="0.2">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -819,25 +824,24 @@
       <c r="H1" s="1" t="s">
         <v>118</v>
       </c>
-      <c r="I1" s="2"/>
-      <c r="J1" s="3"/>
-      <c r="K1" s="3"/>
-      <c r="L1" s="3"/>
-      <c r="M1" s="3"/>
-      <c r="N1" s="3"/>
-      <c r="O1" s="3"/>
-      <c r="P1" s="3"/>
-      <c r="Q1" s="3"/>
-      <c r="R1" s="3"/>
-      <c r="S1" s="3"/>
-      <c r="T1" s="3"/>
-      <c r="U1" s="3"/>
-      <c r="V1" s="3"/>
-      <c r="W1" s="3"/>
-      <c r="X1" s="3"/>
-    </row>
-    <row r="2" spans="1:24" s="1" customFormat="1" x14ac:dyDescent="0.2">
-      <c r="A2" s="4" t="s">
+      <c r="J1" s="2"/>
+      <c r="K1" s="2"/>
+      <c r="L1" s="2"/>
+      <c r="M1" s="2"/>
+      <c r="N1" s="2"/>
+      <c r="O1" s="2"/>
+      <c r="P1" s="2"/>
+      <c r="Q1" s="2"/>
+      <c r="R1" s="2"/>
+      <c r="S1" s="2"/>
+      <c r="T1" s="2"/>
+      <c r="U1" s="2"/>
+      <c r="V1" s="2"/>
+      <c r="W1" s="2"/>
+      <c r="X1" s="2"/>
+    </row>
+    <row r="2" spans="1:24" x14ac:dyDescent="0.2">
+      <c r="A2" s="2" t="s">
         <v>19</v>
       </c>
       <c r="B2" s="1" t="s">
@@ -855,31 +859,31 @@
       <c r="F2" s="1">
         <v>7.3</v>
       </c>
-      <c r="G2" s="4">
+      <c r="G2" s="2">
         <v>2.11</v>
       </c>
       <c r="H2" s="1">
         <v>0.30272596843615496</v>
       </c>
-      <c r="I2" s="3"/>
-      <c r="J2" s="3"/>
-      <c r="K2" s="3"/>
-      <c r="L2" s="3"/>
-      <c r="M2" s="3"/>
-      <c r="N2" s="3"/>
-      <c r="O2" s="3"/>
-      <c r="P2" s="3"/>
-      <c r="Q2" s="3"/>
-      <c r="R2" s="3"/>
-      <c r="S2" s="3"/>
-      <c r="T2" s="3"/>
-      <c r="U2" s="3"/>
-      <c r="V2" s="3"/>
-      <c r="W2" s="3"/>
-      <c r="X2" s="3"/>
-    </row>
-    <row r="3" spans="1:24" s="1" customFormat="1" x14ac:dyDescent="0.2">
-      <c r="A3" s="4" t="s">
+      <c r="I2" s="2"/>
+      <c r="J2" s="2"/>
+      <c r="K2" s="2"/>
+      <c r="L2" s="2"/>
+      <c r="M2" s="2"/>
+      <c r="N2" s="2"/>
+      <c r="O2" s="2"/>
+      <c r="P2" s="2"/>
+      <c r="Q2" s="2"/>
+      <c r="R2" s="2"/>
+      <c r="S2" s="2"/>
+      <c r="T2" s="2"/>
+      <c r="U2" s="2"/>
+      <c r="V2" s="2"/>
+      <c r="W2" s="2"/>
+      <c r="X2" s="2"/>
+    </row>
+    <row r="3" spans="1:24" x14ac:dyDescent="0.2">
+      <c r="A3" s="2" t="s">
         <v>20</v>
       </c>
       <c r="B3" s="1" t="s">
@@ -897,31 +901,16 @@
       <c r="F3" s="1">
         <v>10.1</v>
       </c>
-      <c r="G3" s="4">
+      <c r="G3" s="2">
         <v>2.48</v>
       </c>
       <c r="H3" s="1">
         <v>0.37349397590361449</v>
       </c>
-      <c r="I3" s="3"/>
-      <c r="J3" s="2"/>
-      <c r="K3" s="2"/>
-      <c r="L3" s="2"/>
-      <c r="M3" s="2"/>
-      <c r="N3" s="2"/>
-      <c r="O3" s="2"/>
-      <c r="P3" s="2"/>
-      <c r="Q3" s="2"/>
-      <c r="R3" s="2"/>
-      <c r="S3" s="2"/>
-      <c r="T3" s="2"/>
-      <c r="U3" s="2"/>
-      <c r="V3" s="2"/>
-      <c r="W3" s="2"/>
-      <c r="X3" s="2"/>
-    </row>
-    <row r="4" spans="1:24" s="1" customFormat="1" x14ac:dyDescent="0.2">
-      <c r="A4" s="4" t="s">
+      <c r="I3" s="2"/>
+    </row>
+    <row r="4" spans="1:24" x14ac:dyDescent="0.2">
+      <c r="A4" s="2" t="s">
         <v>21</v>
       </c>
       <c r="B4" s="1" t="s">
@@ -939,31 +928,31 @@
       <c r="F4" s="1">
         <v>7</v>
       </c>
-      <c r="G4" s="4">
+      <c r="G4" s="2">
         <v>1.81</v>
       </c>
       <c r="H4" s="1">
         <v>0.28414442700156989</v>
       </c>
-      <c r="I4" s="3"/>
-      <c r="J4" s="3"/>
-      <c r="K4" s="3"/>
-      <c r="L4" s="3"/>
-      <c r="M4" s="3"/>
-      <c r="N4" s="3"/>
-      <c r="O4" s="3"/>
-      <c r="P4" s="3"/>
-      <c r="Q4" s="3"/>
-      <c r="R4" s="3"/>
-      <c r="S4" s="3"/>
-      <c r="T4" s="3"/>
-      <c r="U4" s="3"/>
-      <c r="V4" s="3"/>
-      <c r="W4" s="3"/>
-      <c r="X4" s="3"/>
-    </row>
-    <row r="5" spans="1:24" s="1" customFormat="1" x14ac:dyDescent="0.2">
-      <c r="A5" s="4" t="s">
+      <c r="I4" s="2"/>
+      <c r="J4" s="2"/>
+      <c r="K4" s="2"/>
+      <c r="L4" s="2"/>
+      <c r="M4" s="2"/>
+      <c r="N4" s="2"/>
+      <c r="O4" s="2"/>
+      <c r="P4" s="2"/>
+      <c r="Q4" s="2"/>
+      <c r="R4" s="2"/>
+      <c r="S4" s="2"/>
+      <c r="T4" s="2"/>
+      <c r="U4" s="2"/>
+      <c r="V4" s="2"/>
+      <c r="W4" s="2"/>
+      <c r="X4" s="2"/>
+    </row>
+    <row r="5" spans="1:24" x14ac:dyDescent="0.2">
+      <c r="A5" s="2" t="s">
         <v>22</v>
       </c>
       <c r="B5" s="1" t="s">
@@ -981,31 +970,15 @@
       <c r="F5" s="1">
         <v>1.3</v>
       </c>
-      <c r="G5" s="4">
+      <c r="G5" s="2">
         <v>2.21</v>
       </c>
       <c r="H5" s="1">
         <v>0.30694444444444441</v>
       </c>
-      <c r="I5" s="2"/>
-      <c r="J5" s="2"/>
-      <c r="K5" s="2"/>
-      <c r="L5" s="2"/>
-      <c r="M5" s="2"/>
-      <c r="N5" s="2"/>
-      <c r="O5" s="2"/>
-      <c r="P5" s="2"/>
-      <c r="Q5" s="2"/>
-      <c r="R5" s="2"/>
-      <c r="S5" s="2"/>
-      <c r="T5" s="2"/>
-      <c r="U5" s="2"/>
-      <c r="V5" s="2"/>
-      <c r="W5" s="2"/>
-      <c r="X5" s="2"/>
-    </row>
-    <row r="6" spans="1:24" s="1" customFormat="1" x14ac:dyDescent="0.2">
-      <c r="A6" s="4" t="s">
+    </row>
+    <row r="6" spans="1:24" x14ac:dyDescent="0.2">
+      <c r="A6" s="2" t="s">
         <v>23</v>
       </c>
       <c r="B6" s="1" t="s">
@@ -1023,31 +996,31 @@
       <c r="F6" s="1">
         <v>4.3</v>
       </c>
-      <c r="G6" s="4">
+      <c r="G6" s="2">
         <v>1.9</v>
       </c>
       <c r="H6" s="1">
         <v>0.28358208955223879</v>
       </c>
-      <c r="I6" s="3"/>
-      <c r="J6" s="3"/>
-      <c r="K6" s="3"/>
-      <c r="L6" s="3"/>
-      <c r="M6" s="3"/>
-      <c r="N6" s="3"/>
-      <c r="O6" s="3"/>
-      <c r="P6" s="3"/>
-      <c r="Q6" s="3"/>
-      <c r="R6" s="3"/>
-      <c r="S6" s="3"/>
-      <c r="T6" s="3"/>
-      <c r="U6" s="3"/>
-      <c r="V6" s="3"/>
-      <c r="W6" s="3"/>
-      <c r="X6" s="3"/>
-    </row>
-    <row r="7" spans="1:24" s="1" customFormat="1" x14ac:dyDescent="0.2">
-      <c r="A7" s="4" t="s">
+      <c r="I6" s="2"/>
+      <c r="J6" s="2"/>
+      <c r="K6" s="2"/>
+      <c r="L6" s="2"/>
+      <c r="M6" s="2"/>
+      <c r="N6" s="2"/>
+      <c r="O6" s="2"/>
+      <c r="P6" s="2"/>
+      <c r="Q6" s="2"/>
+      <c r="R6" s="2"/>
+      <c r="S6" s="2"/>
+      <c r="T6" s="2"/>
+      <c r="U6" s="2"/>
+      <c r="V6" s="2"/>
+      <c r="W6" s="2"/>
+      <c r="X6" s="2"/>
+    </row>
+    <row r="7" spans="1:24" x14ac:dyDescent="0.2">
+      <c r="A7" s="2" t="s">
         <v>24</v>
       </c>
       <c r="B7" s="1" t="s">
@@ -1065,31 +1038,15 @@
       <c r="F7" s="1">
         <v>0.2</v>
       </c>
-      <c r="G7" s="4">
+      <c r="G7" s="2">
         <v>2.34</v>
       </c>
       <c r="H7" s="1">
         <v>0.30310880829015541</v>
       </c>
-      <c r="I7" s="2"/>
-      <c r="J7" s="2"/>
-      <c r="K7" s="2"/>
-      <c r="L7" s="2"/>
-      <c r="M7" s="2"/>
-      <c r="N7" s="2"/>
-      <c r="O7" s="2"/>
-      <c r="P7" s="2"/>
-      <c r="Q7" s="2"/>
-      <c r="R7" s="2"/>
-      <c r="S7" s="2"/>
-      <c r="T7" s="2"/>
-      <c r="U7" s="2"/>
-      <c r="V7" s="2"/>
-      <c r="W7" s="2"/>
-      <c r="X7" s="2"/>
-    </row>
-    <row r="8" spans="1:24" s="1" customFormat="1" x14ac:dyDescent="0.2">
-      <c r="A8" s="4" t="s">
+    </row>
+    <row r="8" spans="1:24" x14ac:dyDescent="0.2">
+      <c r="A8" s="2" t="s">
         <v>25</v>
       </c>
       <c r="B8" s="1" t="s">
@@ -1107,31 +1064,15 @@
       <c r="F8" s="1">
         <v>5.0999999999999996</v>
       </c>
-      <c r="G8" s="4">
+      <c r="G8" s="2">
         <v>2.11</v>
       </c>
       <c r="H8" s="1">
         <v>0.29224376731301938</v>
       </c>
-      <c r="I8" s="2"/>
-      <c r="J8" s="2"/>
-      <c r="K8" s="2"/>
-      <c r="L8" s="2"/>
-      <c r="M8" s="2"/>
-      <c r="N8" s="2"/>
-      <c r="O8" s="2"/>
-      <c r="P8" s="2"/>
-      <c r="Q8" s="2"/>
-      <c r="R8" s="2"/>
-      <c r="S8" s="2"/>
-      <c r="T8" s="2"/>
-      <c r="U8" s="2"/>
-      <c r="V8" s="2"/>
-      <c r="W8" s="2"/>
-      <c r="X8" s="2"/>
-    </row>
-    <row r="9" spans="1:24" s="1" customFormat="1" x14ac:dyDescent="0.2">
-      <c r="A9" s="4" t="s">
+    </row>
+    <row r="9" spans="1:24" x14ac:dyDescent="0.2">
+      <c r="A9" s="2" t="s">
         <v>26</v>
       </c>
       <c r="B9" s="1" t="s">
@@ -1149,31 +1090,15 @@
       <c r="F9" s="1">
         <v>10.4</v>
       </c>
-      <c r="G9" s="4">
+      <c r="G9" s="2">
         <v>2.0499999999999998</v>
       </c>
       <c r="H9" s="1">
         <v>0.33606557377049179</v>
       </c>
-      <c r="I9" s="2"/>
-      <c r="J9" s="2"/>
-      <c r="K9" s="2"/>
-      <c r="L9" s="2"/>
-      <c r="M9" s="2"/>
-      <c r="N9" s="2"/>
-      <c r="O9" s="2"/>
-      <c r="P9" s="2"/>
-      <c r="Q9" s="2"/>
-      <c r="R9" s="2"/>
-      <c r="S9" s="2"/>
-      <c r="T9" s="2"/>
-      <c r="U9" s="2"/>
-      <c r="V9" s="2"/>
-      <c r="W9" s="2"/>
-      <c r="X9" s="2"/>
-    </row>
-    <row r="10" spans="1:24" s="1" customFormat="1" x14ac:dyDescent="0.2">
-      <c r="A10" s="4" t="s">
+    </row>
+    <row r="10" spans="1:24" x14ac:dyDescent="0.2">
+      <c r="A10" s="2" t="s">
         <v>27</v>
       </c>
       <c r="B10" s="1" t="s">
@@ -1191,31 +1116,15 @@
       <c r="F10" s="1">
         <v>9</v>
       </c>
-      <c r="G10" s="4">
+      <c r="G10" s="2">
         <v>1.67</v>
       </c>
       <c r="H10" s="1">
         <v>0.29094076655052264</v>
       </c>
-      <c r="I10" s="2"/>
-      <c r="J10" s="2"/>
-      <c r="K10" s="2"/>
-      <c r="L10" s="2"/>
-      <c r="M10" s="2"/>
-      <c r="N10" s="2"/>
-      <c r="O10" s="2"/>
-      <c r="P10" s="2"/>
-      <c r="Q10" s="2"/>
-      <c r="R10" s="2"/>
-      <c r="S10" s="2"/>
-      <c r="T10" s="2"/>
-      <c r="U10" s="2"/>
-      <c r="V10" s="2"/>
-      <c r="W10" s="2"/>
-      <c r="X10" s="2"/>
-    </row>
-    <row r="11" spans="1:24" s="1" customFormat="1" x14ac:dyDescent="0.2">
-      <c r="A11" s="4" t="s">
+    </row>
+    <row r="11" spans="1:24" x14ac:dyDescent="0.2">
+      <c r="A11" s="2" t="s">
         <v>28</v>
       </c>
       <c r="B11" s="1" t="s">
@@ -1233,31 +1142,15 @@
       <c r="F11" s="1">
         <v>9.5</v>
       </c>
-      <c r="G11" s="4">
+      <c r="G11" s="2">
         <v>1.93</v>
       </c>
       <c r="H11" s="1">
         <v>0.37621832358674462</v>
       </c>
-      <c r="I11" s="2"/>
-      <c r="J11" s="2"/>
-      <c r="K11" s="2"/>
-      <c r="L11" s="2"/>
-      <c r="M11" s="2"/>
-      <c r="N11" s="2"/>
-      <c r="O11" s="2"/>
-      <c r="P11" s="2"/>
-      <c r="Q11" s="2"/>
-      <c r="R11" s="2"/>
-      <c r="S11" s="2"/>
-      <c r="T11" s="2"/>
-      <c r="U11" s="2"/>
-      <c r="V11" s="2"/>
-      <c r="W11" s="2"/>
-      <c r="X11" s="2"/>
-    </row>
-    <row r="12" spans="1:24" s="1" customFormat="1" x14ac:dyDescent="0.2">
-      <c r="A12" s="4" t="s">
+    </row>
+    <row r="12" spans="1:24" x14ac:dyDescent="0.2">
+      <c r="A12" s="2" t="s">
         <v>29</v>
       </c>
       <c r="B12" s="1" t="s">
@@ -1275,31 +1168,15 @@
       <c r="F12" s="1">
         <v>0.4</v>
       </c>
-      <c r="G12" s="4">
+      <c r="G12" s="2">
         <v>1.77</v>
       </c>
       <c r="H12" s="1">
         <v>0.29898648648648651</v>
       </c>
-      <c r="I12" s="2"/>
-      <c r="J12" s="2"/>
-      <c r="K12" s="2"/>
-      <c r="L12" s="2"/>
-      <c r="M12" s="2"/>
-      <c r="N12" s="2"/>
-      <c r="O12" s="2"/>
-      <c r="P12" s="2"/>
-      <c r="Q12" s="2"/>
-      <c r="R12" s="2"/>
-      <c r="S12" s="2"/>
-      <c r="T12" s="2"/>
-      <c r="U12" s="2"/>
-      <c r="V12" s="2"/>
-      <c r="W12" s="2"/>
-      <c r="X12" s="2"/>
-    </row>
-    <row r="13" spans="1:24" s="1" customFormat="1" x14ac:dyDescent="0.2">
-      <c r="A13" s="4" t="s">
+    </row>
+    <row r="13" spans="1:24" x14ac:dyDescent="0.2">
+      <c r="A13" s="2" t="s">
         <v>30</v>
       </c>
       <c r="B13" s="1" t="s">
@@ -1317,31 +1194,15 @@
       <c r="F13" s="1">
         <v>5.5</v>
       </c>
-      <c r="G13" s="4">
+      <c r="G13" s="2">
         <v>1.81</v>
       </c>
       <c r="H13" s="1">
         <v>0.2943089430894309</v>
       </c>
-      <c r="I13" s="2"/>
-      <c r="J13" s="2"/>
-      <c r="K13" s="2"/>
-      <c r="L13" s="2"/>
-      <c r="M13" s="2"/>
-      <c r="N13" s="2"/>
-      <c r="O13" s="2"/>
-      <c r="P13" s="2"/>
-      <c r="Q13" s="2"/>
-      <c r="R13" s="2"/>
-      <c r="S13" s="2"/>
-      <c r="T13" s="2"/>
-      <c r="U13" s="2"/>
-      <c r="V13" s="2"/>
-      <c r="W13" s="2"/>
-      <c r="X13" s="2"/>
-    </row>
-    <row r="14" spans="1:24" s="1" customFormat="1" x14ac:dyDescent="0.2">
-      <c r="A14" s="4" t="s">
+    </row>
+    <row r="14" spans="1:24" x14ac:dyDescent="0.2">
+      <c r="A14" s="2" t="s">
         <v>31</v>
       </c>
       <c r="B14" s="1" t="s">
@@ -1359,31 +1220,15 @@
       <c r="F14" s="1">
         <v>9.1</v>
       </c>
-      <c r="G14" s="4">
+      <c r="G14" s="2">
         <v>2.16</v>
       </c>
       <c r="H14" s="1">
         <v>0.32190760059612522</v>
       </c>
-      <c r="I14" s="2"/>
-      <c r="J14" s="2"/>
-      <c r="K14" s="2"/>
-      <c r="L14" s="2"/>
-      <c r="M14" s="2"/>
-      <c r="N14" s="2"/>
-      <c r="O14" s="2"/>
-      <c r="P14" s="2"/>
-      <c r="Q14" s="2"/>
-      <c r="R14" s="2"/>
-      <c r="S14" s="2"/>
-      <c r="T14" s="2"/>
-      <c r="U14" s="2"/>
-      <c r="V14" s="2"/>
-      <c r="W14" s="2"/>
-      <c r="X14" s="2"/>
-    </row>
-    <row r="15" spans="1:24" s="1" customFormat="1" x14ac:dyDescent="0.2">
-      <c r="A15" s="4" t="s">
+    </row>
+    <row r="15" spans="1:24" x14ac:dyDescent="0.2">
+      <c r="A15" s="2" t="s">
         <v>32</v>
       </c>
       <c r="B15" s="1" t="s">
@@ -1401,31 +1246,15 @@
       <c r="F15" s="1">
         <v>2.1</v>
       </c>
-      <c r="G15" s="4">
+      <c r="G15" s="2">
         <v>2.1</v>
       </c>
       <c r="H15" s="1">
         <v>0.38391224862888479</v>
       </c>
-      <c r="I15" s="2"/>
-      <c r="J15" s="2"/>
-      <c r="K15" s="2"/>
-      <c r="L15" s="2"/>
-      <c r="M15" s="2"/>
-      <c r="N15" s="2"/>
-      <c r="O15" s="2"/>
-      <c r="P15" s="2"/>
-      <c r="Q15" s="2"/>
-      <c r="R15" s="2"/>
-      <c r="S15" s="2"/>
-      <c r="T15" s="2"/>
-      <c r="U15" s="2"/>
-      <c r="V15" s="2"/>
-      <c r="W15" s="2"/>
-      <c r="X15" s="2"/>
-    </row>
-    <row r="16" spans="1:24" s="1" customFormat="1" x14ac:dyDescent="0.2">
-      <c r="A16" s="4" t="s">
+    </row>
+    <row r="16" spans="1:24" x14ac:dyDescent="0.2">
+      <c r="A16" s="2" t="s">
         <v>33</v>
       </c>
       <c r="B16" s="1" t="s">
@@ -1443,31 +1272,16 @@
       <c r="F16" s="1">
         <v>3.5</v>
       </c>
-      <c r="G16" s="4">
+      <c r="G16" s="2">
         <v>1.64</v>
       </c>
       <c r="H16" s="1">
         <v>0.32604373757455268</v>
       </c>
-      <c r="I16" s="2"/>
-      <c r="J16" s="2"/>
-      <c r="K16" s="2"/>
-      <c r="L16" s="2"/>
-      <c r="M16" s="2"/>
-      <c r="N16" s="3"/>
-      <c r="O16" s="2"/>
-      <c r="P16" s="2"/>
-      <c r="Q16" s="2"/>
-      <c r="R16" s="2"/>
-      <c r="S16" s="2"/>
-      <c r="T16" s="2"/>
-      <c r="U16" s="2"/>
-      <c r="V16" s="2"/>
-      <c r="W16" s="2"/>
-      <c r="X16" s="2"/>
-    </row>
-    <row r="17" spans="1:24" s="1" customFormat="1" x14ac:dyDescent="0.2">
-      <c r="A17" s="4" t="s">
+      <c r="N16" s="2"/>
+    </row>
+    <row r="17" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A17" s="2" t="s">
         <v>34</v>
       </c>
       <c r="B17" s="1" t="s">
@@ -1485,31 +1299,15 @@
       <c r="F17" s="1">
         <v>4.5</v>
       </c>
-      <c r="G17" s="4">
+      <c r="G17" s="2">
         <v>2.23</v>
       </c>
       <c r="H17" s="1">
         <v>0.42884615384615382</v>
       </c>
-      <c r="I17" s="2"/>
-      <c r="J17" s="2"/>
-      <c r="K17" s="2"/>
-      <c r="L17" s="2"/>
-      <c r="M17" s="2"/>
-      <c r="N17" s="2"/>
-      <c r="O17" s="2"/>
-      <c r="P17" s="2"/>
-      <c r="Q17" s="2"/>
-      <c r="R17" s="2"/>
-      <c r="S17" s="2"/>
-      <c r="T17" s="2"/>
-      <c r="U17" s="2"/>
-      <c r="V17" s="2"/>
-      <c r="W17" s="2"/>
-      <c r="X17" s="2"/>
-    </row>
-    <row r="18" spans="1:24" s="1" customFormat="1" x14ac:dyDescent="0.2">
-      <c r="A18" s="4" t="s">
+    </row>
+    <row r="18" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A18" s="2" t="s">
         <v>35</v>
       </c>
       <c r="B18" s="1" t="s">
@@ -1527,31 +1325,15 @@
       <c r="F18" s="1">
         <v>5.6</v>
       </c>
-      <c r="G18" s="4">
+      <c r="G18" s="2">
         <v>1.88</v>
       </c>
       <c r="H18" s="1">
         <v>0.3949579831932773</v>
       </c>
-      <c r="I18" s="2"/>
-      <c r="J18" s="2"/>
-      <c r="K18" s="2"/>
-      <c r="L18" s="2"/>
-      <c r="M18" s="2"/>
-      <c r="N18" s="2"/>
-      <c r="O18" s="2"/>
-      <c r="P18" s="2"/>
-      <c r="Q18" s="2"/>
-      <c r="R18" s="2"/>
-      <c r="S18" s="2"/>
-      <c r="T18" s="2"/>
-      <c r="U18" s="2"/>
-      <c r="V18" s="2"/>
-      <c r="W18" s="2"/>
-      <c r="X18" s="2"/>
-    </row>
-    <row r="19" spans="1:24" s="1" customFormat="1" x14ac:dyDescent="0.2">
-      <c r="A19" s="4" t="s">
+    </row>
+    <row r="19" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A19" s="2" t="s">
         <v>36</v>
       </c>
       <c r="B19" s="1" t="s">
@@ -1569,15 +1351,15 @@
       <c r="F19" s="1">
         <v>3.5</v>
       </c>
-      <c r="G19" s="4">
+      <c r="G19" s="2">
         <v>1.52</v>
       </c>
       <c r="H19" s="1">
         <v>0.33187772925764192</v>
       </c>
     </row>
-    <row r="20" spans="1:24" s="1" customFormat="1" x14ac:dyDescent="0.2">
-      <c r="A20" s="4" t="s">
+    <row r="20" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A20" s="2" t="s">
         <v>37</v>
       </c>
       <c r="B20" s="1" t="s">
@@ -1595,15 +1377,15 @@
       <c r="F20" s="1">
         <v>3.2</v>
       </c>
-      <c r="G20" s="4">
+      <c r="G20" s="2">
         <v>1.54</v>
       </c>
       <c r="H20" s="1">
         <v>0.28838951310861427</v>
       </c>
     </row>
-    <row r="21" spans="1:24" s="1" customFormat="1" x14ac:dyDescent="0.2">
-      <c r="A21" s="4" t="s">
+    <row r="21" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A21" s="2" t="s">
         <v>38</v>
       </c>
       <c r="B21" s="1" t="s">
@@ -1621,15 +1403,15 @@
       <c r="F21" s="1">
         <v>3.9</v>
       </c>
-      <c r="G21" s="4">
+      <c r="G21" s="2">
         <v>1.53</v>
       </c>
       <c r="H21" s="1">
         <v>0.32484076433121017</v>
       </c>
     </row>
-    <row r="22" spans="1:24" s="1" customFormat="1" x14ac:dyDescent="0.2">
-      <c r="A22" s="4" t="s">
+    <row r="22" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A22" s="2" t="s">
         <v>39</v>
       </c>
       <c r="B22" s="1" t="s">
@@ -1647,15 +1429,15 @@
       <c r="F22" s="1">
         <v>7.9</v>
       </c>
-      <c r="G22" s="4">
+      <c r="G22" s="2">
         <v>2.0299999999999998</v>
       </c>
       <c r="H22" s="1">
         <v>0.44130434782608696</v>
       </c>
     </row>
-    <row r="23" spans="1:24" s="1" customFormat="1" x14ac:dyDescent="0.2">
-      <c r="A23" s="4" t="s">
+    <row r="23" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A23" s="2" t="s">
         <v>40</v>
       </c>
       <c r="B23" s="1" t="s">
@@ -1673,15 +1455,15 @@
       <c r="F23" s="1">
         <v>6.1</v>
       </c>
-      <c r="G23" s="4">
+      <c r="G23" s="2">
         <v>1.91</v>
       </c>
       <c r="H23" s="1">
         <v>0.35239852398523985</v>
       </c>
     </row>
-    <row r="24" spans="1:24" s="1" customFormat="1" x14ac:dyDescent="0.2">
-      <c r="A24" s="4" t="s">
+    <row r="24" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A24" s="2" t="s">
         <v>41</v>
       </c>
       <c r="B24" s="1" t="s">
@@ -1699,15 +1481,15 @@
       <c r="F24" s="1">
         <v>3.9</v>
       </c>
-      <c r="G24" s="4">
+      <c r="G24" s="2">
         <v>1.83</v>
       </c>
       <c r="H24" s="1">
         <v>0.27853881278538817</v>
       </c>
     </row>
-    <row r="25" spans="1:24" s="1" customFormat="1" x14ac:dyDescent="0.2">
-      <c r="A25" s="4" t="s">
+    <row r="25" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A25" s="2" t="s">
         <v>42</v>
       </c>
       <c r="B25" s="1" t="s">
@@ -1725,15 +1507,15 @@
       <c r="F25" s="1">
         <v>3.6</v>
       </c>
-      <c r="G25" s="4">
+      <c r="G25" s="2">
         <v>2.38</v>
       </c>
       <c r="H25" s="1">
         <v>0.3005050505050505</v>
       </c>
     </row>
-    <row r="26" spans="1:24" s="1" customFormat="1" x14ac:dyDescent="0.2">
-      <c r="A26" s="4" t="s">
+    <row r="26" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A26" s="2" t="s">
         <v>43</v>
       </c>
       <c r="B26" s="1" t="s">
@@ -1751,15 +1533,15 @@
       <c r="F26" s="1">
         <v>1.2</v>
       </c>
-      <c r="G26" s="4">
+      <c r="G26" s="2">
         <v>1.41</v>
       </c>
       <c r="H26" s="1">
         <v>0.24780316344463973</v>
       </c>
     </row>
-    <row r="27" spans="1:24" s="1" customFormat="1" x14ac:dyDescent="0.2">
-      <c r="A27" s="4" t="s">
+    <row r="27" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A27" s="2" t="s">
         <v>44</v>
       </c>
       <c r="B27" s="1" t="s">
@@ -1777,15 +1559,15 @@
       <c r="F27" s="1">
         <v>2.7</v>
       </c>
-      <c r="G27" s="4">
+      <c r="G27" s="2">
         <v>1.43</v>
       </c>
       <c r="H27" s="1">
         <v>0.25176056338028169</v>
       </c>
     </row>
-    <row r="28" spans="1:24" s="1" customFormat="1" x14ac:dyDescent="0.2">
-      <c r="A28" s="4" t="s">
+    <row r="28" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A28" s="2" t="s">
         <v>45</v>
       </c>
       <c r="B28" s="1" t="s">
@@ -1803,15 +1585,15 @@
       <c r="F28" s="1">
         <v>1.1000000000000001</v>
       </c>
-      <c r="G28" s="4">
+      <c r="G28" s="2">
         <v>1.73</v>
       </c>
       <c r="H28" s="1">
         <v>0.2831423895253683</v>
       </c>
     </row>
-    <row r="29" spans="1:24" s="1" customFormat="1" x14ac:dyDescent="0.2">
-      <c r="A29" s="4" t="s">
+    <row r="29" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A29" s="2" t="s">
         <v>46</v>
       </c>
       <c r="B29" s="1" t="s">
@@ -1829,15 +1611,15 @@
       <c r="F29" s="1">
         <v>2.1</v>
       </c>
-      <c r="G29" s="4">
+      <c r="G29" s="2">
         <v>1.87</v>
       </c>
       <c r="H29" s="1">
         <v>0.28205128205128205</v>
       </c>
     </row>
-    <row r="30" spans="1:24" s="1" customFormat="1" x14ac:dyDescent="0.2">
-      <c r="A30" s="4" t="s">
+    <row r="30" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A30" s="2" t="s">
         <v>47</v>
       </c>
       <c r="B30" s="1" t="s">
@@ -1855,15 +1637,15 @@
       <c r="F30" s="1">
         <v>7</v>
       </c>
-      <c r="G30" s="4">
+      <c r="G30" s="2">
         <v>1.65</v>
       </c>
       <c r="H30" s="1">
         <v>0.32480314960629919</v>
       </c>
     </row>
-    <row r="31" spans="1:24" s="1" customFormat="1" x14ac:dyDescent="0.2">
-      <c r="A31" s="4" t="s">
+    <row r="31" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A31" s="2" t="s">
         <v>48</v>
       </c>
       <c r="B31" s="1" t="s">
@@ -1881,15 +1663,15 @@
       <c r="F31" s="1">
         <v>6.5</v>
       </c>
-      <c r="G31" s="4">
+      <c r="G31" s="2">
         <v>0.98</v>
       </c>
       <c r="H31" s="1">
         <v>0.29080118694362017</v>
       </c>
     </row>
-    <row r="32" spans="1:24" s="1" customFormat="1" x14ac:dyDescent="0.2">
-      <c r="A32" s="4" t="s">
+    <row r="32" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A32" s="2" t="s">
         <v>49</v>
       </c>
       <c r="B32" s="1" t="s">
@@ -1907,15 +1689,15 @@
       <c r="F32" s="1">
         <v>1.1000000000000001</v>
       </c>
-      <c r="G32" s="4">
+      <c r="G32" s="2">
         <v>2.27</v>
       </c>
       <c r="H32" s="1">
         <v>0.29634464751958223</v>
       </c>
     </row>
-    <row r="33" spans="1:8" s="1" customFormat="1" x14ac:dyDescent="0.2">
-      <c r="A33" s="4" t="s">
+    <row r="33" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A33" s="2" t="s">
         <v>50</v>
       </c>
       <c r="B33" s="1" t="s">
@@ -1933,15 +1715,15 @@
       <c r="F33" s="1">
         <v>6.1</v>
       </c>
-      <c r="G33" s="4">
+      <c r="G33" s="2">
         <v>1.44</v>
       </c>
       <c r="H33" s="1">
         <v>0.27639155470249521</v>
       </c>
     </row>
-    <row r="34" spans="1:8" s="1" customFormat="1" x14ac:dyDescent="0.2">
-      <c r="A34" s="4" t="s">
+    <row r="34" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A34" s="2" t="s">
         <v>51</v>
       </c>
       <c r="B34" s="1" t="s">
@@ -1959,15 +1741,15 @@
       <c r="F34" s="1">
         <v>5.2</v>
       </c>
-      <c r="G34" s="4">
+      <c r="G34" s="2">
         <v>2.0299999999999998</v>
       </c>
       <c r="H34" s="1">
         <v>0.29765395894428148</v>
       </c>
     </row>
-    <row r="35" spans="1:8" s="1" customFormat="1" x14ac:dyDescent="0.2">
-      <c r="A35" s="4" t="s">
+    <row r="35" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A35" s="2" t="s">
         <v>52</v>
       </c>
       <c r="B35" s="1" t="s">
@@ -1985,15 +1767,15 @@
       <c r="F35" s="1">
         <v>3.5</v>
       </c>
-      <c r="G35" s="4">
+      <c r="G35" s="2">
         <v>2.0299999999999998</v>
       </c>
       <c r="H35" s="1">
         <v>0.30208333333333331</v>
       </c>
     </row>
-    <row r="36" spans="1:8" s="1" customFormat="1" x14ac:dyDescent="0.2">
-      <c r="A36" s="4" t="s">
+    <row r="36" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A36" s="2" t="s">
         <v>53</v>
       </c>
       <c r="B36" s="1" t="s">
@@ -2011,15 +1793,15 @@
       <c r="F36" s="1">
         <v>4.8</v>
       </c>
-      <c r="G36" s="4">
+      <c r="G36" s="2">
         <v>1.84</v>
       </c>
       <c r="H36" s="1">
         <v>0.32508833922261482</v>
       </c>
     </row>
-    <row r="37" spans="1:8" s="1" customFormat="1" x14ac:dyDescent="0.2">
-      <c r="A37" s="4" t="s">
+    <row r="37" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A37" s="2" t="s">
         <v>54</v>
       </c>
       <c r="B37" s="1" t="s">
@@ -2037,15 +1819,15 @@
       <c r="F37" s="1">
         <v>13.7</v>
       </c>
-      <c r="G37" s="4">
+      <c r="G37" s="2">
         <v>0.87</v>
       </c>
       <c r="H37" s="1">
         <v>0.22081218274111675</v>
       </c>
     </row>
-    <row r="38" spans="1:8" s="1" customFormat="1" x14ac:dyDescent="0.2">
-      <c r="A38" s="4" t="s">
+    <row r="38" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A38" s="2" t="s">
         <v>55</v>
       </c>
       <c r="B38" s="1" t="s">
@@ -2063,15 +1845,15 @@
       <c r="F38" s="1">
         <v>4.0999999999999996</v>
       </c>
-      <c r="G38" s="4">
+      <c r="G38" s="2">
         <v>1.49</v>
       </c>
       <c r="H38" s="1">
         <v>0.30532786885245899</v>
       </c>
     </row>
-    <row r="39" spans="1:8" s="1" customFormat="1" x14ac:dyDescent="0.2">
-      <c r="A39" s="4" t="s">
+    <row r="39" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A39" s="2" t="s">
         <v>56</v>
       </c>
       <c r="B39" s="1" t="s">
@@ -2089,15 +1871,15 @@
       <c r="F39" s="1">
         <v>4.2</v>
       </c>
-      <c r="G39" s="4">
+      <c r="G39" s="2">
         <v>1.8</v>
       </c>
       <c r="H39" s="1">
         <v>0.29315960912052119</v>
       </c>
     </row>
-    <row r="40" spans="1:8" s="1" customFormat="1" x14ac:dyDescent="0.2">
-      <c r="A40" s="4" t="s">
+    <row r="40" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A40" s="2" t="s">
         <v>57</v>
       </c>
       <c r="B40" s="1" t="s">
@@ -2115,15 +1897,15 @@
       <c r="F40" s="1">
         <v>5.7</v>
       </c>
-      <c r="G40" s="4">
+      <c r="G40" s="2">
         <v>2.7</v>
       </c>
       <c r="H40" s="1">
         <v>0.33582089552238814</v>
       </c>
     </row>
-    <row r="41" spans="1:8" s="1" customFormat="1" x14ac:dyDescent="0.2">
-      <c r="A41" s="4" t="s">
+    <row r="41" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A41" s="2" t="s">
         <v>58</v>
       </c>
       <c r="B41" s="1" t="s">
@@ -2141,15 +1923,15 @@
       <c r="F41" s="1">
         <v>2.4</v>
       </c>
-      <c r="G41" s="4">
+      <c r="G41" s="2">
         <v>1.66</v>
       </c>
       <c r="H41" s="1">
         <v>0.25382262996941896</v>
       </c>
     </row>
-    <row r="42" spans="1:8" s="1" customFormat="1" x14ac:dyDescent="0.2">
-      <c r="A42" s="4" t="s">
+    <row r="42" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A42" s="2" t="s">
         <v>59</v>
       </c>
       <c r="B42" s="1" t="s">
@@ -2167,15 +1949,15 @@
       <c r="F42" s="1">
         <v>8.5</v>
       </c>
-      <c r="G42" s="4">
+      <c r="G42" s="2">
         <v>1.47</v>
       </c>
       <c r="H42" s="1">
         <v>0.31887201735357923</v>
       </c>
     </row>
-    <row r="43" spans="1:8" s="1" customFormat="1" x14ac:dyDescent="0.2">
-      <c r="A43" s="4" t="s">
+    <row r="43" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A43" s="2" t="s">
         <v>60</v>
       </c>
       <c r="B43" s="1" t="s">
@@ -2193,15 +1975,15 @@
       <c r="F43" s="1">
         <v>6.6</v>
       </c>
-      <c r="G43" s="4">
+      <c r="G43" s="2">
         <v>1.21</v>
       </c>
       <c r="H43" s="1">
         <v>0.25854700854700857</v>
       </c>
     </row>
-    <row r="44" spans="1:8" s="1" customFormat="1" x14ac:dyDescent="0.2">
-      <c r="A44" s="4" t="s">
+    <row r="44" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A44" s="2" t="s">
         <v>61</v>
       </c>
       <c r="B44" s="1" t="s">
@@ -2219,15 +2001,15 @@
       <c r="F44" s="1">
         <v>8</v>
       </c>
-      <c r="G44" s="4">
+      <c r="G44" s="2">
         <v>0.95</v>
       </c>
       <c r="H44" s="1">
         <v>0.19709543568464727</v>
       </c>
     </row>
-    <row r="45" spans="1:8" s="1" customFormat="1" x14ac:dyDescent="0.2">
-      <c r="A45" s="4" t="s">
+    <row r="45" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A45" s="2" t="s">
         <v>62</v>
       </c>
       <c r="B45" s="1" t="s">
@@ -2245,15 +2027,15 @@
       <c r="F45" s="1">
         <v>2.7</v>
       </c>
-      <c r="G45" s="4">
+      <c r="G45" s="2">
         <v>0.75</v>
       </c>
       <c r="H45" s="1">
         <v>0.14734774066797643</v>
       </c>
     </row>
-    <row r="46" spans="1:8" s="1" customFormat="1" x14ac:dyDescent="0.2">
-      <c r="A46" s="4" t="s">
+    <row r="46" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A46" s="2" t="s">
         <v>63</v>
       </c>
       <c r="B46" s="1" t="s">
@@ -2271,15 +2053,15 @@
       <c r="F46" s="1">
         <v>17.5</v>
       </c>
-      <c r="G46" s="4">
+      <c r="G46" s="2">
         <v>1.25</v>
       </c>
       <c r="H46" s="1">
         <v>0.29411764705882354</v>
       </c>
     </row>
-    <row r="47" spans="1:8" s="1" customFormat="1" x14ac:dyDescent="0.2">
-      <c r="A47" s="4" t="s">
+    <row r="47" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A47" s="2" t="s">
         <v>64</v>
       </c>
       <c r="B47" s="1" t="s">
@@ -2297,15 +2079,15 @@
       <c r="F47" s="1">
         <v>12.2</v>
       </c>
-      <c r="G47" s="4">
+      <c r="G47" s="2">
         <v>0.61</v>
       </c>
       <c r="H47" s="1">
         <v>0.21554770318021199</v>
       </c>
     </row>
-    <row r="48" spans="1:8" s="1" customFormat="1" x14ac:dyDescent="0.2">
-      <c r="A48" s="4" t="s">
+    <row r="48" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A48" s="2" t="s">
         <v>65</v>
       </c>
       <c r="B48" s="1" t="s">
@@ -2323,15 +2105,15 @@
       <c r="F48" s="1">
         <v>-0.2</v>
       </c>
-      <c r="G48" s="4">
+      <c r="G48" s="2">
         <v>2.0499999999999998</v>
       </c>
       <c r="H48" s="1">
         <v>0.26147959183673469</v>
       </c>
     </row>
-    <row r="49" spans="1:8" s="1" customFormat="1" x14ac:dyDescent="0.2">
-      <c r="A49" s="4" t="s">
+    <row r="49" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A49" s="2" t="s">
         <v>66</v>
       </c>
       <c r="B49" s="1" t="s">
@@ -2349,15 +2131,15 @@
       <c r="F49" s="1">
         <v>9</v>
       </c>
-      <c r="G49" s="4">
+      <c r="G49" s="2">
         <v>1.07</v>
       </c>
       <c r="H49" s="1">
         <v>0.32035928143712578</v>
       </c>
     </row>
-    <row r="50" spans="1:8" s="1" customFormat="1" x14ac:dyDescent="0.2">
-      <c r="A50" s="4" t="s">
+    <row r="50" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A50" s="2" t="s">
         <v>67</v>
       </c>
       <c r="B50" s="1" t="s">
@@ -2375,15 +2157,15 @@
       <c r="F50" s="1">
         <v>0.3</v>
       </c>
-      <c r="G50" s="4">
+      <c r="G50" s="2">
         <v>2.37</v>
       </c>
       <c r="H50" s="1">
         <v>0.33521923620933525</v>
       </c>
     </row>
-    <row r="51" spans="1:8" s="1" customFormat="1" x14ac:dyDescent="0.2">
-      <c r="A51" s="4" t="s">
+    <row r="51" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A51" s="2" t="s">
         <v>68</v>
       </c>
       <c r="B51" s="1" t="s">
@@ -2401,15 +2183,15 @@
       <c r="F51" s="1">
         <v>1.7</v>
       </c>
-      <c r="G51" s="4">
+      <c r="G51" s="2">
         <v>1.88</v>
       </c>
       <c r="H51" s="1">
         <v>0.27089337175792505</v>
       </c>
     </row>
-    <row r="52" spans="1:8" s="1" customFormat="1" x14ac:dyDescent="0.2">
-      <c r="A52" s="4" t="s">
+    <row r="52" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A52" s="2" t="s">
         <v>69</v>
       </c>
       <c r="B52" s="1" t="s">
@@ -2427,15 +2209,15 @@
       <c r="F52" s="1">
         <v>3.1</v>
       </c>
-      <c r="G52" s="4">
+      <c r="G52" s="2">
         <v>1.93</v>
       </c>
       <c r="H52" s="1">
         <v>0.31331168831168832</v>
       </c>
     </row>
-    <row r="53" spans="1:8" s="1" customFormat="1" x14ac:dyDescent="0.2">
-      <c r="A53" s="4" t="s">
+    <row r="53" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A53" s="2" t="s">
         <v>70</v>
       </c>
       <c r="B53" s="1" t="s">
@@ -2453,15 +2235,15 @@
       <c r="F53" s="1">
         <v>0.8</v>
       </c>
-      <c r="G53" s="4">
+      <c r="G53" s="2">
         <v>1.44</v>
       </c>
       <c r="H53" s="1">
         <v>0.22052067381317</v>
       </c>
     </row>
-    <row r="54" spans="1:8" s="1" customFormat="1" x14ac:dyDescent="0.2">
-      <c r="A54" s="4" t="s">
+    <row r="54" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A54" s="2" t="s">
         <v>71</v>
       </c>
       <c r="B54" s="1" t="s">
@@ -2479,15 +2261,15 @@
       <c r="F54" s="1">
         <v>3.2</v>
       </c>
-      <c r="G54" s="4">
+      <c r="G54" s="2">
         <v>2.02</v>
       </c>
       <c r="H54" s="1">
         <v>0.30467571644042235</v>
       </c>
     </row>
-    <row r="55" spans="1:8" s="1" customFormat="1" x14ac:dyDescent="0.2">
-      <c r="A55" s="4" t="s">
+    <row r="55" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A55" s="2" t="s">
         <v>72</v>
       </c>
       <c r="B55" s="1" t="s">
@@ -2505,15 +2287,15 @@
       <c r="F55" s="1">
         <v>11.2</v>
       </c>
-      <c r="G55" s="4">
+      <c r="G55" s="2">
         <v>1.4</v>
       </c>
       <c r="H55" s="1">
         <v>0.24911032028469748</v>
       </c>
     </row>
-    <row r="56" spans="1:8" s="1" customFormat="1" x14ac:dyDescent="0.2">
-      <c r="A56" s="4" t="s">
+    <row r="56" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A56" s="2" t="s">
         <v>73</v>
       </c>
       <c r="B56" s="1" t="s">
@@ -2531,15 +2313,15 @@
       <c r="F56" s="1">
         <v>12.3</v>
       </c>
-      <c r="G56" s="4">
+      <c r="G56" s="2">
         <v>1.1000000000000001</v>
       </c>
       <c r="H56" s="1">
         <v>0.27160493827160498</v>
       </c>
     </row>
-    <row r="57" spans="1:8" s="1" customFormat="1" x14ac:dyDescent="0.2">
-      <c r="A57" s="4" t="s">
+    <row r="57" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A57" s="2" t="s">
         <v>74</v>
       </c>
       <c r="B57" s="1" t="s">
@@ -2557,15 +2339,15 @@
       <c r="F57" s="1">
         <v>7.1</v>
       </c>
-      <c r="G57" s="4">
+      <c r="G57" s="2">
         <v>1.71</v>
       </c>
       <c r="H57" s="1">
         <v>0.33075435203094777</v>
       </c>
     </row>
-    <row r="58" spans="1:8" s="1" customFormat="1" x14ac:dyDescent="0.2">
-      <c r="A58" s="4" t="s">
+    <row r="58" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A58" s="2" t="s">
         <v>75</v>
       </c>
       <c r="B58" s="1" t="s">
@@ -2583,15 +2365,15 @@
       <c r="F58" s="1">
         <v>0.6</v>
       </c>
-      <c r="G58" s="4">
+      <c r="G58" s="2">
         <v>0.66</v>
       </c>
       <c r="H58" s="1">
         <v>0.12222222222222222</v>
       </c>
     </row>
-    <row r="59" spans="1:8" s="1" customFormat="1" x14ac:dyDescent="0.2">
-      <c r="A59" s="4" t="s">
+    <row r="59" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A59" s="2" t="s">
         <v>76</v>
       </c>
       <c r="B59" s="1" t="s">
@@ -2609,15 +2391,15 @@
       <c r="F59" s="1">
         <v>3.2</v>
       </c>
-      <c r="G59" s="4">
+      <c r="G59" s="2">
         <v>1.73</v>
       </c>
       <c r="H59" s="1">
         <v>0.27503974562798089</v>
       </c>
     </row>
-    <row r="60" spans="1:8" s="1" customFormat="1" x14ac:dyDescent="0.2">
-      <c r="A60" s="4" t="s">
+    <row r="60" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A60" s="2" t="s">
         <v>77</v>
       </c>
       <c r="B60" s="1" t="s">
@@ -2635,15 +2417,15 @@
       <c r="F60" s="1">
         <v>8.1999999999999993</v>
       </c>
-      <c r="G60" s="4">
+      <c r="G60" s="2">
         <v>2.0699999999999998</v>
       </c>
       <c r="H60" s="1">
         <v>0.25618811881188119</v>
       </c>
     </row>
-    <row r="61" spans="1:8" s="1" customFormat="1" x14ac:dyDescent="0.2">
-      <c r="A61" s="4" t="s">
+    <row r="61" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A61" s="2" t="s">
         <v>78</v>
       </c>
       <c r="B61" s="1" t="s">
@@ -2661,15 +2443,15 @@
       <c r="F61" s="1">
         <v>7</v>
       </c>
-      <c r="G61" s="4">
+      <c r="G61" s="2">
         <v>1.61</v>
       </c>
       <c r="H61" s="1">
         <v>0.24769230769230771</v>
       </c>
     </row>
-    <row r="62" spans="1:8" s="1" customFormat="1" x14ac:dyDescent="0.2">
-      <c r="A62" s="4" t="s">
+    <row r="62" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A62" s="2" t="s">
         <v>79</v>
       </c>
       <c r="B62" s="1" t="s">
@@ -2687,15 +2469,15 @@
       <c r="F62" s="1">
         <v>0.2</v>
       </c>
-      <c r="G62" s="4">
+      <c r="G62" s="2">
         <v>1.68</v>
       </c>
       <c r="H62" s="1">
         <v>0.24172661870503598</v>
       </c>
     </row>
-    <row r="63" spans="1:8" s="1" customFormat="1" x14ac:dyDescent="0.2">
-      <c r="A63" s="4" t="s">
+    <row r="63" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A63" s="2" t="s">
         <v>80</v>
       </c>
       <c r="B63" s="1" t="s">
@@ -2713,15 +2495,15 @@
       <c r="F63" s="1">
         <v>1.3</v>
       </c>
-      <c r="G63" s="4">
+      <c r="G63" s="2">
         <v>1.69</v>
       </c>
       <c r="H63" s="1">
         <v>0.26242236024844723</v>
       </c>
     </row>
-    <row r="64" spans="1:8" s="1" customFormat="1" x14ac:dyDescent="0.2">
-      <c r="A64" s="4" t="s">
+    <row r="64" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A64" s="2" t="s">
         <v>81</v>
       </c>
       <c r="B64" s="1" t="s">
@@ -2739,15 +2521,15 @@
       <c r="F64" s="1">
         <v>1.1000000000000001</v>
       </c>
-      <c r="G64" s="4">
+      <c r="G64" s="2">
         <v>2.02</v>
       </c>
       <c r="H64" s="1">
         <v>0.27297297297297296</v>
       </c>
     </row>
-    <row r="65" spans="1:8" s="1" customFormat="1" x14ac:dyDescent="0.2">
-      <c r="A65" s="4" t="s">
+    <row r="65" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A65" s="2" t="s">
         <v>82</v>
       </c>
       <c r="B65" s="1" t="s">
@@ -2765,15 +2547,15 @@
       <c r="F65" s="1">
         <v>6.5</v>
       </c>
-      <c r="G65" s="4">
+      <c r="G65" s="2">
         <v>1.1599999999999999</v>
       </c>
       <c r="H65" s="1">
         <v>0.22745098039215686</v>
       </c>
     </row>
-    <row r="66" spans="1:8" s="1" customFormat="1" x14ac:dyDescent="0.2">
-      <c r="A66" s="4" t="s">
+    <row r="66" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A66" s="2" t="s">
         <v>83</v>
       </c>
       <c r="B66" s="1" t="s">
@@ -2791,15 +2573,15 @@
       <c r="F66" s="1">
         <v>14.2</v>
       </c>
-      <c r="G66" s="4">
+      <c r="G66" s="2">
         <v>1.63</v>
       </c>
       <c r="H66" s="1">
         <v>0.34315789473684211</v>
       </c>
     </row>
-    <row r="67" spans="1:8" s="1" customFormat="1" x14ac:dyDescent="0.2">
-      <c r="A67" s="4" t="s">
+    <row r="67" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A67" s="2" t="s">
         <v>84</v>
       </c>
       <c r="B67" s="1" t="s">
@@ -2817,15 +2599,15 @@
       <c r="F67" s="1">
         <v>15.5</v>
       </c>
-      <c r="G67" s="4">
+      <c r="G67" s="2">
         <v>1.58</v>
       </c>
       <c r="H67" s="1">
         <v>0.33545647558386416</v>
       </c>
     </row>
-    <row r="68" spans="1:8" s="1" customFormat="1" x14ac:dyDescent="0.2">
-      <c r="A68" s="4" t="s">
+    <row r="68" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A68" s="2" t="s">
         <v>85</v>
       </c>
       <c r="B68" s="1" t="s">
@@ -2843,15 +2625,15 @@
       <c r="F68" s="1">
         <v>12.1</v>
       </c>
-      <c r="G68" s="4">
+      <c r="G68" s="2">
         <v>1.68</v>
       </c>
       <c r="H68" s="1">
         <v>0.3</v>
       </c>
     </row>
-    <row r="69" spans="1:8" s="1" customFormat="1" x14ac:dyDescent="0.2">
-      <c r="A69" s="4" t="s">
+    <row r="69" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A69" s="2" t="s">
         <v>86</v>
       </c>
       <c r="B69" s="1" t="s">
@@ -2869,15 +2651,15 @@
       <c r="F69" s="1">
         <v>12.8</v>
       </c>
-      <c r="G69" s="4">
+      <c r="G69" s="2">
         <v>1.67</v>
       </c>
       <c r="H69" s="1">
         <v>0.34647302904564314</v>
       </c>
     </row>
-    <row r="70" spans="1:8" s="1" customFormat="1" x14ac:dyDescent="0.2">
-      <c r="A70" s="4" t="s">
+    <row r="70" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A70" s="2" t="s">
         <v>87</v>
       </c>
       <c r="B70" s="1" t="s">
@@ -2895,15 +2677,15 @@
       <c r="F70" s="1">
         <v>16.899999999999999</v>
       </c>
-      <c r="G70" s="4">
+      <c r="G70" s="2">
         <v>0.9</v>
       </c>
       <c r="H70" s="1">
         <v>0.3461538461538462</v>
       </c>
     </row>
-    <row r="71" spans="1:8" s="1" customFormat="1" x14ac:dyDescent="0.2">
-      <c r="A71" s="4" t="s">
+    <row r="71" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A71" s="2" t="s">
         <v>88</v>
       </c>
       <c r="B71" s="1" t="s">
@@ -2921,15 +2703,15 @@
       <c r="F71" s="1">
         <v>6.8</v>
       </c>
-      <c r="G71" s="4">
+      <c r="G71" s="2">
         <v>0.82</v>
       </c>
       <c r="H71" s="1">
         <v>0.20603015075376885</v>
       </c>
     </row>
-    <row r="72" spans="1:8" s="1" customFormat="1" x14ac:dyDescent="0.2">
-      <c r="A72" s="4" t="s">
+    <row r="72" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A72" s="2" t="s">
         <v>89</v>
       </c>
       <c r="B72" s="1" t="s">
@@ -2947,15 +2729,15 @@
       <c r="F72" s="1">
         <v>8.3000000000000007</v>
       </c>
-      <c r="G72" s="4">
+      <c r="G72" s="2">
         <v>1.68</v>
       </c>
       <c r="H72" s="1">
         <v>0.3428571428571428</v>
       </c>
     </row>
-    <row r="73" spans="1:8" s="1" customFormat="1" x14ac:dyDescent="0.2">
-      <c r="A73" s="4" t="s">
+    <row r="73" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A73" s="2" t="s">
         <v>90</v>
       </c>
       <c r="B73" s="1" t="s">
@@ -2973,15 +2755,15 @@
       <c r="F73" s="1">
         <v>13.4</v>
       </c>
-      <c r="G73" s="4">
+      <c r="G73" s="2">
         <v>1.2</v>
       </c>
       <c r="H73" s="1">
         <v>0.32171581769436997</v>
       </c>
     </row>
-    <row r="74" spans="1:8" s="1" customFormat="1" x14ac:dyDescent="0.2">
-      <c r="A74" s="4" t="s">
+    <row r="74" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A74" s="2" t="s">
         <v>91</v>
       </c>
       <c r="B74" s="1" t="s">
@@ -2999,15 +2781,15 @@
       <c r="F74" s="1">
         <v>8.1999999999999993</v>
       </c>
-      <c r="G74" s="4">
+      <c r="G74" s="2">
         <v>2.7</v>
       </c>
       <c r="H74" s="1">
         <v>0.39073806078147616</v>
       </c>
     </row>
-    <row r="75" spans="1:8" s="1" customFormat="1" x14ac:dyDescent="0.2">
-      <c r="A75" s="4" t="s">
+    <row r="75" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A75" s="2" t="s">
         <v>92</v>
       </c>
       <c r="B75" s="1" t="s">
@@ -3025,15 +2807,15 @@
       <c r="F75" s="1">
         <v>11.9</v>
       </c>
-      <c r="G75" s="4">
+      <c r="G75" s="2">
         <v>1.4</v>
       </c>
       <c r="H75" s="1">
         <v>0.30837004405286339</v>
       </c>
     </row>
-    <row r="76" spans="1:8" s="1" customFormat="1" x14ac:dyDescent="0.2">
-      <c r="A76" s="4" t="s">
+    <row r="76" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A76" s="2" t="s">
         <v>93</v>
       </c>
       <c r="B76" s="1" t="s">
@@ -3051,15 +2833,15 @@
       <c r="F76" s="1">
         <v>8.3000000000000007</v>
       </c>
-      <c r="G76" s="4">
+      <c r="G76" s="2">
         <v>0.76</v>
       </c>
       <c r="H76" s="1">
         <v>0.19740259740259741</v>
       </c>
     </row>
-    <row r="77" spans="1:8" s="1" customFormat="1" x14ac:dyDescent="0.2">
-      <c r="A77" s="4" t="s">
+    <row r="77" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A77" s="2" t="s">
         <v>94</v>
       </c>
       <c r="B77" s="1" t="s">
@@ -3077,15 +2859,15 @@
       <c r="F77" s="1">
         <v>9.5</v>
       </c>
-      <c r="G77" s="4">
+      <c r="G77" s="2">
         <v>0.9</v>
       </c>
       <c r="H77" s="1">
         <v>0.20881670533642691</v>
       </c>
     </row>
-    <row r="78" spans="1:8" s="1" customFormat="1" x14ac:dyDescent="0.2">
-      <c r="A78" s="4" t="s">
+    <row r="78" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A78" s="2" t="s">
         <v>95</v>
       </c>
       <c r="B78" s="1" t="s">
@@ -3103,15 +2885,15 @@
       <c r="F78" s="1">
         <v>8.4</v>
       </c>
-      <c r="G78" s="4">
+      <c r="G78" s="2">
         <v>1.4</v>
       </c>
       <c r="H78" s="1">
         <v>0.30368763557483736</v>
       </c>
     </row>
-    <row r="79" spans="1:8" s="1" customFormat="1" x14ac:dyDescent="0.2">
-      <c r="A79" s="4" t="s">
+    <row r="79" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A79" s="2" t="s">
         <v>96</v>
       </c>
       <c r="B79" s="1" t="s">
@@ -3129,15 +2911,15 @@
       <c r="F79" s="1">
         <v>2.4</v>
       </c>
-      <c r="G79" s="4">
+      <c r="G79" s="2">
         <v>1.74</v>
       </c>
       <c r="H79" s="1">
         <v>0.27315541601255888</v>
       </c>
     </row>
-    <row r="80" spans="1:8" s="1" customFormat="1" x14ac:dyDescent="0.2">
-      <c r="A80" s="4" t="s">
+    <row r="80" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A80" s="2" t="s">
         <v>97</v>
       </c>
       <c r="B80" s="1" t="s">
@@ -3155,15 +2937,15 @@
       <c r="F80" s="1">
         <v>0</v>
       </c>
-      <c r="G80" s="4">
+      <c r="G80" s="2">
         <v>2.0499999999999998</v>
       </c>
       <c r="H80" s="1">
         <v>0.31782945736434109</v>
       </c>
     </row>
-    <row r="81" spans="1:8" s="1" customFormat="1" x14ac:dyDescent="0.2">
-      <c r="A81" s="4" t="s">
+    <row r="81" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A81" s="2" t="s">
         <v>98</v>
       </c>
       <c r="B81" s="1" t="s">
@@ -3181,15 +2963,15 @@
       <c r="F81" s="1">
         <v>7</v>
       </c>
-      <c r="G81" s="4">
+      <c r="G81" s="2">
         <v>2.06</v>
       </c>
       <c r="H81" s="1">
         <v>0.30700447093889716</v>
       </c>
     </row>
-    <row r="82" spans="1:8" s="1" customFormat="1" x14ac:dyDescent="0.2">
-      <c r="A82" s="4" t="s">
+    <row r="82" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A82" s="2" t="s">
         <v>99</v>
       </c>
       <c r="B82" s="1" t="s">
@@ -3207,15 +2989,15 @@
       <c r="F82" s="1">
         <v>5.3</v>
       </c>
-      <c r="G82" s="4">
+      <c r="G82" s="2">
         <v>1.93</v>
       </c>
       <c r="H82" s="1">
         <v>0.30634920634920637</v>
       </c>
     </row>
-    <row r="83" spans="1:8" s="1" customFormat="1" x14ac:dyDescent="0.2">
-      <c r="A83" s="4" t="s">
+    <row r="83" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A83" s="2" t="s">
         <v>100</v>
       </c>
       <c r="B83" s="1" t="s">
@@ -3233,15 +3015,15 @@
       <c r="F83" s="1">
         <v>3.6</v>
       </c>
-      <c r="G83" s="4">
+      <c r="G83" s="2">
         <v>1.35</v>
       </c>
       <c r="H83" s="1">
         <v>0.31177829099307158</v>
       </c>
     </row>
-    <row r="84" spans="1:8" s="1" customFormat="1" x14ac:dyDescent="0.2">
-      <c r="A84" s="4" t="s">
+    <row r="84" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A84" s="2" t="s">
         <v>101</v>
       </c>
       <c r="B84" s="1" t="s">
@@ -3259,15 +3041,15 @@
       <c r="F84" s="1">
         <v>2.4</v>
       </c>
-      <c r="G84" s="4">
+      <c r="G84" s="2">
         <v>1.85</v>
       </c>
       <c r="H84" s="1">
         <v>0.30228758169934644</v>
       </c>
     </row>
-    <row r="85" spans="1:8" s="1" customFormat="1" x14ac:dyDescent="0.2">
-      <c r="A85" s="4" t="s">
+    <row r="85" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A85" s="2" t="s">
         <v>102</v>
       </c>
       <c r="B85" s="1" t="s">
@@ -3285,15 +3067,15 @@
       <c r="F85" s="1">
         <v>1.7</v>
       </c>
-      <c r="G85" s="4">
+      <c r="G85" s="2">
         <v>1.1000000000000001</v>
       </c>
       <c r="H85" s="1">
         <v>0.16666666666666669</v>
       </c>
     </row>
-    <row r="86" spans="1:8" s="1" customFormat="1" x14ac:dyDescent="0.2">
-      <c r="A86" s="4" t="s">
+    <row r="86" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A86" s="2" t="s">
         <v>103</v>
       </c>
       <c r="B86" s="1" t="s">
@@ -3311,15 +3093,15 @@
       <c r="F86" s="1">
         <v>1.2</v>
       </c>
-      <c r="G86" s="4">
+      <c r="G86" s="2">
         <v>1.97</v>
       </c>
       <c r="H86" s="1">
         <v>0.27707454289732775</v>
       </c>
     </row>
-    <row r="87" spans="1:8" s="1" customFormat="1" x14ac:dyDescent="0.2">
-      <c r="A87" s="4" t="s">
+    <row r="87" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A87" s="2" t="s">
         <v>104</v>
       </c>
       <c r="B87" s="1" t="s">
@@ -3337,15 +3119,15 @@
       <c r="F87" s="1">
         <v>6.2</v>
       </c>
-      <c r="G87" s="4">
+      <c r="G87" s="2">
         <v>1.21</v>
       </c>
       <c r="H87" s="1">
         <v>0.20473773265651438</v>
       </c>
     </row>
-    <row r="88" spans="1:8" s="1" customFormat="1" x14ac:dyDescent="0.2">
-      <c r="A88" s="4" t="s">
+    <row r="88" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A88" s="2" t="s">
         <v>105</v>
       </c>
       <c r="B88" s="1" t="s">
@@ -3363,15 +3145,15 @@
       <c r="F88" s="1">
         <v>4.9000000000000004</v>
       </c>
-      <c r="G88" s="4">
+      <c r="G88" s="2">
         <v>0.87</v>
       </c>
       <c r="H88" s="1">
         <v>0.14974182444061962</v>
       </c>
     </row>
-    <row r="89" spans="1:8" s="1" customFormat="1" x14ac:dyDescent="0.2">
-      <c r="A89" s="4" t="s">
+    <row r="89" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A89" s="2" t="s">
         <v>106</v>
       </c>
       <c r="B89" s="1" t="s">
@@ -3389,15 +3171,15 @@
       <c r="F89" s="1">
         <v>3.6</v>
       </c>
-      <c r="G89" s="4">
+      <c r="G89" s="2">
         <v>1.73</v>
       </c>
       <c r="H89" s="1">
         <v>0.27768860353130015</v>
       </c>
     </row>
-    <row r="90" spans="1:8" s="1" customFormat="1" x14ac:dyDescent="0.2">
-      <c r="A90" s="4" t="s">
+    <row r="90" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A90" s="2" t="s">
         <v>107</v>
       </c>
       <c r="B90" s="1" t="s">
@@ -3415,15 +3197,15 @@
       <c r="F90" s="1">
         <v>4</v>
       </c>
-      <c r="G90" s="4">
+      <c r="G90" s="2">
         <v>1.61</v>
       </c>
       <c r="H90" s="1">
         <v>0.27288135593220342</v>
       </c>
     </row>
-    <row r="91" spans="1:8" s="1" customFormat="1" x14ac:dyDescent="0.2">
-      <c r="A91" s="4" t="s">
+    <row r="91" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A91" s="2" t="s">
         <v>108</v>
       </c>
       <c r="B91" s="1" t="s">
@@ -3441,15 +3223,15 @@
       <c r="F91" s="1">
         <v>6</v>
       </c>
-      <c r="G91" s="4">
+      <c r="G91" s="2">
         <v>1.33</v>
       </c>
       <c r="H91" s="1">
         <v>0.25094339622641509</v>
       </c>
     </row>
-    <row r="92" spans="1:8" s="1" customFormat="1" x14ac:dyDescent="0.2">
-      <c r="A92" s="4" t="s">
+    <row r="92" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A92" s="2" t="s">
         <v>109</v>
       </c>
       <c r="B92" s="1" t="s">
@@ -3467,15 +3249,15 @@
       <c r="F92" s="1">
         <v>6.7</v>
       </c>
-      <c r="G92" s="4">
+      <c r="G92" s="2">
         <v>0.6</v>
       </c>
       <c r="H92" s="1">
         <v>0.11881188118811881</v>
       </c>
     </row>
-    <row r="93" spans="1:8" s="1" customFormat="1" x14ac:dyDescent="0.2">
-      <c r="A93" s="4" t="s">
+    <row r="93" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A93" s="2" t="s">
         <v>110</v>
       </c>
       <c r="B93" s="1" t="s">
@@ -3493,15 +3275,15 @@
       <c r="F93" s="1">
         <v>10.8</v>
       </c>
-      <c r="G93" s="4">
+      <c r="G93" s="2">
         <v>1.0900000000000001</v>
       </c>
       <c r="H93" s="1">
         <v>0.2395604395604396</v>
       </c>
     </row>
-    <row r="94" spans="1:8" s="1" customFormat="1" x14ac:dyDescent="0.2">
-      <c r="A94" s="4" t="s">
+    <row r="94" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A94" s="2" t="s">
         <v>111</v>
       </c>
       <c r="B94" s="1" t="s">
@@ -3519,15 +3301,15 @@
       <c r="F94" s="1">
         <v>3.6</v>
       </c>
-      <c r="G94" s="4">
+      <c r="G94" s="2">
         <v>1.42</v>
       </c>
       <c r="H94" s="1">
         <v>0.20285714285714285</v>
       </c>
     </row>
-    <row r="95" spans="1:8" s="1" customFormat="1" x14ac:dyDescent="0.2">
-      <c r="A95" s="4" t="s">
+    <row r="95" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A95" s="2" t="s">
         <v>112</v>
       </c>
       <c r="B95" s="1" t="s">
@@ -3545,15 +3327,15 @@
       <c r="F95" s="1">
         <v>2.2999999999999998</v>
       </c>
-      <c r="G95" s="4">
+      <c r="G95" s="2">
         <v>1.1599999999999999</v>
       </c>
       <c r="H95" s="1">
         <v>0.16338028169014082</v>
       </c>
     </row>
-    <row r="96" spans="1:8" s="1" customFormat="1" x14ac:dyDescent="0.2">
-      <c r="A96" s="4" t="s">
+    <row r="96" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A96" s="2" t="s">
         <v>113</v>
       </c>
       <c r="B96" s="1" t="s">
@@ -3571,15 +3353,15 @@
       <c r="F96" s="1">
         <v>5</v>
       </c>
-      <c r="G96" s="4">
+      <c r="G96" s="2">
         <v>1.01</v>
       </c>
       <c r="H96" s="1">
         <v>0.18498168498168499</v>
       </c>
     </row>
-    <row r="97" spans="1:8" s="1" customFormat="1" x14ac:dyDescent="0.2">
-      <c r="A97" s="4" t="s">
+    <row r="97" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A97" s="2" t="s">
         <v>114</v>
       </c>
       <c r="B97" s="1" t="s">
@@ -3597,15 +3379,15 @@
       <c r="F97" s="1">
         <v>6.5</v>
       </c>
-      <c r="G97" s="4">
+      <c r="G97" s="2">
         <v>1.04</v>
       </c>
       <c r="H97" s="1">
         <v>0.17508417508417509</v>
       </c>
     </row>
-    <row r="98" spans="1:8" s="1" customFormat="1" x14ac:dyDescent="0.2">
-      <c r="A98" s="4" t="s">
+    <row r="98" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A98" s="2" t="s">
         <v>115</v>
       </c>
       <c r="B98" s="1" t="s">
@@ -3623,15 +3405,15 @@
       <c r="F98" s="1">
         <v>7.7</v>
       </c>
-      <c r="G98" s="4">
+      <c r="G98" s="2">
         <v>1.35</v>
       </c>
       <c r="H98" s="1">
         <v>0.27551020408163263</v>
       </c>
     </row>
-    <row r="99" spans="1:8" s="1" customFormat="1" x14ac:dyDescent="0.2">
-      <c r="A99" s="4" t="s">
+    <row r="99" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A99" s="2" t="s">
         <v>116</v>
       </c>
       <c r="B99" s="1" t="s">
@@ -3649,14 +3431,14 @@
       <c r="F99" s="1">
         <v>1.5</v>
       </c>
-      <c r="G99" s="4">
+      <c r="G99" s="2">
         <v>0.88</v>
       </c>
       <c r="H99" s="1">
         <v>0.1461794019933555</v>
       </c>
     </row>
-    <row r="100" spans="1:8" s="1" customFormat="1" x14ac:dyDescent="0.2">
+    <row r="100" spans="1:8" x14ac:dyDescent="0.2">
       <c r="G100" s="1">
         <f>MAX(G2:G99)</f>
         <v>2.7</v>

</xml_diff>

<commit_message>
Updated statistical methods and scripts.
</commit_message>
<xml_diff>
--- a/2025greenhouse/2025greenhousemaster.xlsx
+++ b/2025greenhouse/2025greenhousemaster.xlsx
@@ -1,27 +1,20 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10215"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10322"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/reneedavis/R/Biobead/2025greenhouse/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E0E29788-C20D-EE44-9942-A5A86D2D3A31}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5BF89B58-E641-2749-9CC4-2F9F4EB8727D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="1060" yWindow="920" windowWidth="25260" windowHeight="15800" xr2:uid="{F83686B1-B1F8-0E46-8563-14D114C6B912}"/>
   </bookViews>
   <sheets>
     <sheet name="Master" sheetId="1" r:id="rId1"/>
   </sheets>
-  <definedNames>
-    <definedName name="_xlchart.v1.0" hidden="1">Master!$C$2:$C$99</definedName>
-    <definedName name="_xlchart.v1.1" hidden="1">Master!$H$2:$H$99</definedName>
-    <definedName name="_xlchart.v1.2" hidden="1">Master!$H$2:$H$99</definedName>
-    <definedName name="_xlchart.v1.3" hidden="1">Master!$F$2:$F$99</definedName>
-    <definedName name="_xlchart.v1.4" hidden="1">Master!$F$2:$F$99</definedName>
-  </definedNames>
   <calcPr calcId="191029"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
@@ -43,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="204" uniqueCount="120">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="206" uniqueCount="122">
   <si>
     <t>Sample_ID</t>
   </si>
@@ -403,13 +396,19 @@
   </si>
   <si>
     <t>GrainWeight_g</t>
+  </si>
+  <si>
+    <t>AMF_colonization</t>
+  </si>
+  <si>
+    <t>Root_Shoot</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="3" x14ac:knownFonts="1">
+  <fonts count="4" x14ac:knownFonts="1">
     <font>
       <sz val="12"/>
       <color theme="1"/>
@@ -428,6 +427,12 @@
       <color rgb="FF000000"/>
       <name val="Aptos Narrow"/>
       <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <color rgb="FF000000"/>
+      <name val="Helvetica Neue"/>
+      <family val="2"/>
     </font>
   </fonts>
   <fills count="2">
@@ -450,10 +455,11 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -788,7 +794,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{5F4F35E3-E0A7-C644-BFF1-CE1B44684279}">
-  <dimension ref="A1:X100"/>
+  <dimension ref="A1:X99"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="10.83203125" style="1"/>
@@ -796,7 +802,8 @@
     <col min="3" max="6" width="10.83203125" style="1"/>
     <col min="7" max="7" width="10.5" style="1" bestFit="1" customWidth="1"/>
     <col min="8" max="8" width="12.6640625" style="1" bestFit="1" customWidth="1"/>
-    <col min="9" max="16384" width="10.83203125" style="1"/>
+    <col min="9" max="9" width="10.83203125" style="1"/>
+    <col min="11" max="16384" width="10.83203125" style="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:24" x14ac:dyDescent="0.2">
@@ -824,7 +831,12 @@
       <c r="H1" s="1" t="s">
         <v>118</v>
       </c>
-      <c r="J1" s="2"/>
+      <c r="I1" s="3" t="s">
+        <v>120</v>
+      </c>
+      <c r="J1" t="s">
+        <v>121</v>
+      </c>
       <c r="K1" s="2"/>
       <c r="L1" s="2"/>
       <c r="M1" s="2"/>
@@ -865,8 +877,12 @@
       <c r="H2" s="1">
         <v>0.30272596843615496</v>
       </c>
-      <c r="I2" s="2"/>
-      <c r="J2" s="2"/>
+      <c r="I2" s="3">
+        <v>54.901960799999998</v>
+      </c>
+      <c r="J2">
+        <v>0.15638450500000001</v>
+      </c>
       <c r="K2" s="2"/>
       <c r="L2" s="2"/>
       <c r="M2" s="2"/>
@@ -907,7 +923,12 @@
       <c r="H3" s="1">
         <v>0.37349397590361449</v>
       </c>
-      <c r="I3" s="2"/>
+      <c r="I3" s="3">
+        <v>60.194174799999999</v>
+      </c>
+      <c r="J3">
+        <v>0.12801204799999999</v>
+      </c>
     </row>
     <row r="4" spans="1:24" x14ac:dyDescent="0.2">
       <c r="A4" s="2" t="s">
@@ -934,8 +955,12 @@
       <c r="H4" s="1">
         <v>0.28414442700156989</v>
       </c>
-      <c r="I4" s="2"/>
-      <c r="J4" s="2"/>
+      <c r="I4" s="3">
+        <v>66.346153799999996</v>
+      </c>
+      <c r="J4">
+        <v>0.188383046</v>
+      </c>
       <c r="K4" s="2"/>
       <c r="L4" s="2"/>
       <c r="M4" s="2"/>
@@ -976,6 +1001,12 @@
       <c r="H5" s="1">
         <v>0.30694444444444441</v>
       </c>
+      <c r="I5" s="3">
+        <v>38.655462200000002</v>
+      </c>
+      <c r="J5">
+        <v>0.17222222200000001</v>
+      </c>
     </row>
     <row r="6" spans="1:24" x14ac:dyDescent="0.2">
       <c r="A6" s="2" t="s">
@@ -1002,8 +1033,12 @@
       <c r="H6" s="1">
         <v>0.28358208955223879</v>
       </c>
-      <c r="I6" s="2"/>
-      <c r="J6" s="2"/>
+      <c r="I6" s="3">
+        <v>40.776699000000001</v>
+      </c>
+      <c r="J6">
+        <v>0.173134328</v>
+      </c>
       <c r="K6" s="2"/>
       <c r="L6" s="2"/>
       <c r="M6" s="2"/>
@@ -1044,6 +1079,12 @@
       <c r="H7" s="1">
         <v>0.30310880829015541</v>
       </c>
+      <c r="I7" s="3">
+        <v>58.823529399999998</v>
+      </c>
+      <c r="J7">
+        <v>0.183937824</v>
+      </c>
     </row>
     <row r="8" spans="1:24" x14ac:dyDescent="0.2">
       <c r="A8" s="2" t="s">
@@ -1070,6 +1111,12 @@
       <c r="H8" s="1">
         <v>0.29224376731301938</v>
       </c>
+      <c r="I8" s="3">
+        <v>54.285714300000002</v>
+      </c>
+      <c r="J8">
+        <v>0.200831025</v>
+      </c>
     </row>
     <row r="9" spans="1:24" x14ac:dyDescent="0.2">
       <c r="A9" s="2" t="s">
@@ -1096,6 +1143,12 @@
       <c r="H9" s="1">
         <v>0.33606557377049179</v>
       </c>
+      <c r="I9" s="3">
+        <v>69</v>
+      </c>
+      <c r="J9">
+        <v>0.16393442599999999</v>
+      </c>
     </row>
     <row r="10" spans="1:24" x14ac:dyDescent="0.2">
       <c r="A10" s="2" t="s">
@@ -1122,6 +1175,12 @@
       <c r="H10" s="1">
         <v>0.29094076655052264</v>
       </c>
+      <c r="I10" s="3">
+        <v>56.862745099999998</v>
+      </c>
+      <c r="J10">
+        <v>0.18466899000000001</v>
+      </c>
     </row>
     <row r="11" spans="1:24" x14ac:dyDescent="0.2">
       <c r="A11" s="2" t="s">
@@ -1148,6 +1207,12 @@
       <c r="H11" s="1">
         <v>0.37621832358674462</v>
       </c>
+      <c r="I11" s="3">
+        <v>66.666666699999993</v>
+      </c>
+      <c r="J11">
+        <v>0.233918129</v>
+      </c>
     </row>
     <row r="12" spans="1:24" x14ac:dyDescent="0.2">
       <c r="A12" s="2" t="s">
@@ -1174,6 +1239,12 @@
       <c r="H12" s="1">
         <v>0.29898648648648651</v>
       </c>
+      <c r="I12" s="3">
+        <v>71.698113199999995</v>
+      </c>
+      <c r="J12">
+        <v>0.18243243200000001</v>
+      </c>
     </row>
     <row r="13" spans="1:24" x14ac:dyDescent="0.2">
       <c r="A13" s="2" t="s">
@@ -1200,6 +1271,12 @@
       <c r="H13" s="1">
         <v>0.2943089430894309</v>
       </c>
+      <c r="I13" s="3">
+        <v>60.194174799999999</v>
+      </c>
+      <c r="J13">
+        <v>0.144715447</v>
+      </c>
     </row>
     <row r="14" spans="1:24" x14ac:dyDescent="0.2">
       <c r="A14" s="2" t="s">
@@ -1226,6 +1303,12 @@
       <c r="H14" s="1">
         <v>0.32190760059612522</v>
       </c>
+      <c r="I14" s="3">
+        <v>68</v>
+      </c>
+      <c r="J14">
+        <v>0.180327869</v>
+      </c>
     </row>
     <row r="15" spans="1:24" x14ac:dyDescent="0.2">
       <c r="A15" s="2" t="s">
@@ -1252,6 +1335,12 @@
       <c r="H15" s="1">
         <v>0.38391224862888479</v>
       </c>
+      <c r="I15" s="3">
+        <v>66.019417500000003</v>
+      </c>
+      <c r="J15">
+        <v>0.20840950599999999</v>
+      </c>
     </row>
     <row r="16" spans="1:24" x14ac:dyDescent="0.2">
       <c r="A16" s="2" t="s">
@@ -1278,9 +1367,15 @@
       <c r="H16" s="1">
         <v>0.32604373757455268</v>
       </c>
+      <c r="I16" s="3">
+        <v>46.280991700000001</v>
+      </c>
+      <c r="J16">
+        <v>0.25646123300000001</v>
+      </c>
       <c r="N16" s="2"/>
     </row>
-    <row r="17" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="17" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A17" s="2" t="s">
         <v>34</v>
       </c>
@@ -1305,8 +1400,14 @@
       <c r="H17" s="1">
         <v>0.42884615384615382</v>
       </c>
-    </row>
-    <row r="18" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="I17" s="3">
+        <v>65</v>
+      </c>
+      <c r="J17">
+        <v>0.25</v>
+      </c>
+    </row>
+    <row r="18" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A18" s="2" t="s">
         <v>35</v>
       </c>
@@ -1331,8 +1432,14 @@
       <c r="H18" s="1">
         <v>0.3949579831932773</v>
       </c>
-    </row>
-    <row r="19" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="I18" s="3">
+        <v>63.725490200000003</v>
+      </c>
+      <c r="J18">
+        <v>0.19327731100000001</v>
+      </c>
+    </row>
+    <row r="19" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A19" s="2" t="s">
         <v>36</v>
       </c>
@@ -1357,8 +1464,14 @@
       <c r="H19" s="1">
         <v>0.33187772925764192</v>
       </c>
-    </row>
-    <row r="20" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="I19" s="3">
+        <v>63.461538500000003</v>
+      </c>
+      <c r="J19">
+        <v>0.18340611400000001</v>
+      </c>
+    </row>
+    <row r="20" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A20" s="2" t="s">
         <v>37</v>
       </c>
@@ -1383,8 +1496,14 @@
       <c r="H20" s="1">
         <v>0.28838951310861427</v>
       </c>
-    </row>
-    <row r="21" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="I20" s="3">
+        <v>71.428571399999996</v>
+      </c>
+      <c r="J20">
+        <v>0.234082397</v>
+      </c>
+    </row>
+    <row r="21" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A21" s="2" t="s">
         <v>38</v>
       </c>
@@ -1409,8 +1528,14 @@
       <c r="H21" s="1">
         <v>0.32484076433121017</v>
       </c>
-    </row>
-    <row r="22" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="I21" s="3">
+        <v>62.264150899999997</v>
+      </c>
+      <c r="J21">
+        <v>0.18895966</v>
+      </c>
+    </row>
+    <row r="22" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A22" s="2" t="s">
         <v>39</v>
       </c>
@@ -1435,8 +1560,14 @@
       <c r="H22" s="1">
         <v>0.44130434782608696</v>
       </c>
-    </row>
-    <row r="23" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="I22" s="3">
+        <v>62.962963000000002</v>
+      </c>
+      <c r="J22">
+        <v>0.22608695700000001</v>
+      </c>
+    </row>
+    <row r="23" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A23" s="2" t="s">
         <v>40</v>
       </c>
@@ -1461,8 +1592,14 @@
       <c r="H23" s="1">
         <v>0.35239852398523985</v>
       </c>
-    </row>
-    <row r="24" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="I23" s="3">
+        <v>68.224299099999996</v>
+      </c>
+      <c r="J23">
+        <v>0.19557195599999999</v>
+      </c>
+    </row>
+    <row r="24" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A24" s="2" t="s">
         <v>41</v>
       </c>
@@ -1487,8 +1624,14 @@
       <c r="H24" s="1">
         <v>0.27853881278538817</v>
       </c>
-    </row>
-    <row r="25" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="I24" s="3">
+        <v>67.857142899999999</v>
+      </c>
+      <c r="J24">
+        <v>0.27245053299999999</v>
+      </c>
+    </row>
+    <row r="25" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A25" s="2" t="s">
         <v>42</v>
       </c>
@@ -1513,8 +1656,14 @@
       <c r="H25" s="1">
         <v>0.3005050505050505</v>
       </c>
-    </row>
-    <row r="26" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="I25" s="3">
+        <v>57.692307700000001</v>
+      </c>
+      <c r="J25">
+        <v>0.20959596</v>
+      </c>
+    </row>
+    <row r="26" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A26" s="2" t="s">
         <v>43</v>
       </c>
@@ -1539,8 +1688,14 @@
       <c r="H26" s="1">
         <v>0.24780316344463973</v>
       </c>
-    </row>
-    <row r="27" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="I26" s="3">
+        <v>79.710144900000003</v>
+      </c>
+      <c r="J26">
+        <v>0.22144112499999999</v>
+      </c>
+    </row>
+    <row r="27" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A27" s="2" t="s">
         <v>44</v>
       </c>
@@ -1565,8 +1720,14 @@
       <c r="H27" s="1">
         <v>0.25176056338028169</v>
       </c>
-    </row>
-    <row r="28" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="I27" s="3">
+        <v>68.224299099999996</v>
+      </c>
+      <c r="J27">
+        <v>0.22183098600000001</v>
+      </c>
+    </row>
+    <row r="28" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A28" s="2" t="s">
         <v>45</v>
       </c>
@@ -1591,8 +1752,14 @@
       <c r="H28" s="1">
         <v>0.2831423895253683</v>
       </c>
-    </row>
-    <row r="29" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="I28" s="3">
+        <v>61.165048499999997</v>
+      </c>
+      <c r="J28">
+        <v>0.240589198</v>
+      </c>
+    </row>
+    <row r="29" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A29" s="2" t="s">
         <v>46</v>
       </c>
@@ -1617,8 +1784,14 @@
       <c r="H29" s="1">
         <v>0.28205128205128205</v>
       </c>
-    </row>
-    <row r="30" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="I29" s="3">
+        <v>55.454545500000002</v>
+      </c>
+      <c r="J29">
+        <v>0.26696832599999998</v>
+      </c>
+    </row>
+    <row r="30" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A30" s="2" t="s">
         <v>47</v>
       </c>
@@ -1643,8 +1816,14 @@
       <c r="H30" s="1">
         <v>0.32480314960629919</v>
       </c>
-    </row>
-    <row r="31" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="I30" s="3">
+        <v>59.813084099999998</v>
+      </c>
+      <c r="J30">
+        <v>0.155511811</v>
+      </c>
+    </row>
+    <row r="31" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A31" s="2" t="s">
         <v>48</v>
       </c>
@@ -1669,8 +1848,14 @@
       <c r="H31" s="1">
         <v>0.29080118694362017</v>
       </c>
-    </row>
-    <row r="32" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="I31" s="3">
+        <v>48.1481481</v>
+      </c>
+      <c r="J31">
+        <v>0.25519287800000001</v>
+      </c>
+    </row>
+    <row r="32" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A32" s="2" t="s">
         <v>49</v>
       </c>
@@ -1695,8 +1880,14 @@
       <c r="H32" s="1">
         <v>0.29634464751958223</v>
       </c>
-    </row>
-    <row r="33" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="I32" s="3">
+        <v>57</v>
+      </c>
+      <c r="J32">
+        <v>0.24020887699999999</v>
+      </c>
+    </row>
+    <row r="33" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A33" s="2" t="s">
         <v>50</v>
       </c>
@@ -1721,8 +1912,14 @@
       <c r="H33" s="1">
         <v>0.27639155470249521</v>
       </c>
-    </row>
-    <row r="34" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="I33" s="3">
+        <v>56.730769199999997</v>
+      </c>
+      <c r="J33">
+        <v>0.21689059499999999</v>
+      </c>
+    </row>
+    <row r="34" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A34" s="2" t="s">
         <v>51</v>
       </c>
@@ -1747,8 +1944,14 @@
       <c r="H34" s="1">
         <v>0.29765395894428148</v>
       </c>
-    </row>
-    <row r="35" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="I34" s="3">
+        <v>58.3333333</v>
+      </c>
+      <c r="J34">
+        <v>0.19354838699999999</v>
+      </c>
+    </row>
+    <row r="35" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A35" s="2" t="s">
         <v>52</v>
       </c>
@@ -1773,8 +1976,14 @@
       <c r="H35" s="1">
         <v>0.30208333333333331</v>
       </c>
-    </row>
-    <row r="36" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="I35" s="3">
+        <v>51.968503900000002</v>
+      </c>
+      <c r="J35">
+        <v>0.171130952</v>
+      </c>
+    </row>
+    <row r="36" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A36" s="2" t="s">
         <v>53</v>
       </c>
@@ -1799,8 +2008,14 @@
       <c r="H36" s="1">
         <v>0.32508833922261482</v>
       </c>
-    </row>
-    <row r="37" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="I36" s="3">
+        <v>49.5049505</v>
+      </c>
+      <c r="J36">
+        <v>0.247349823</v>
+      </c>
+    </row>
+    <row r="37" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A37" s="2" t="s">
         <v>54</v>
       </c>
@@ -1825,8 +2040,14 @@
       <c r="H37" s="1">
         <v>0.22081218274111675</v>
       </c>
-    </row>
-    <row r="38" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="I37" s="3">
+        <v>60.169491499999999</v>
+      </c>
+      <c r="J37">
+        <v>0.15482233500000001</v>
+      </c>
+    </row>
+    <row r="38" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A38" s="2" t="s">
         <v>55</v>
       </c>
@@ -1851,8 +2072,14 @@
       <c r="H38" s="1">
         <v>0.30532786885245899</v>
       </c>
-    </row>
-    <row r="39" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="I38" s="3">
+        <v>53.968254000000002</v>
+      </c>
+      <c r="J38">
+        <v>0.159836066</v>
+      </c>
+    </row>
+    <row r="39" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A39" s="2" t="s">
         <v>56</v>
       </c>
@@ -1877,8 +2104,14 @@
       <c r="H39" s="1">
         <v>0.29315960912052119</v>
       </c>
-    </row>
-    <row r="40" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="I39" s="3">
+        <v>68.965517199999994</v>
+      </c>
+      <c r="J39">
+        <v>0.166123779</v>
+      </c>
+    </row>
+    <row r="40" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A40" s="2" t="s">
         <v>57</v>
       </c>
@@ -1903,8 +2136,14 @@
       <c r="H40" s="1">
         <v>0.33582089552238814</v>
       </c>
-    </row>
-    <row r="41" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="I40" s="3">
+        <v>56.637168099999997</v>
+      </c>
+      <c r="J40">
+        <v>0.16417910399999999</v>
+      </c>
+    </row>
+    <row r="41" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A41" s="2" t="s">
         <v>58</v>
       </c>
@@ -1929,8 +2168,14 @@
       <c r="H41" s="1">
         <v>0.25382262996941896</v>
       </c>
-    </row>
-    <row r="42" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="I41" s="3">
+        <v>57.03125</v>
+      </c>
+      <c r="J41">
+        <v>0.172782875</v>
+      </c>
+    </row>
+    <row r="42" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A42" s="2" t="s">
         <v>59</v>
       </c>
@@ -1955,8 +2200,14 @@
       <c r="H42" s="1">
         <v>0.31887201735357923</v>
       </c>
-    </row>
-    <row r="43" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="I42" s="3">
+        <v>56.410256400000002</v>
+      </c>
+      <c r="J42">
+        <v>0.154013015</v>
+      </c>
+    </row>
+    <row r="43" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A43" s="2" t="s">
         <v>60</v>
       </c>
@@ -1981,8 +2232,14 @@
       <c r="H43" s="1">
         <v>0.25854700854700857</v>
       </c>
-    </row>
-    <row r="44" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="I43" s="3">
+        <v>49.180327900000002</v>
+      </c>
+      <c r="J43">
+        <v>0.213675214</v>
+      </c>
+    </row>
+    <row r="44" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A44" s="2" t="s">
         <v>61</v>
       </c>
@@ -2007,8 +2264,14 @@
       <c r="H44" s="1">
         <v>0.19709543568464727</v>
       </c>
-    </row>
-    <row r="45" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="I44" s="3">
+        <v>39.252336399999997</v>
+      </c>
+      <c r="J44">
+        <v>0.16390041499999999</v>
+      </c>
+    </row>
+    <row r="45" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A45" s="2" t="s">
         <v>62</v>
       </c>
@@ -2033,8 +2296,14 @@
       <c r="H45" s="1">
         <v>0.14734774066797643</v>
       </c>
-    </row>
-    <row r="46" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="I45" s="3">
+        <v>38.596491200000003</v>
+      </c>
+      <c r="J45">
+        <v>0.26129666000000001</v>
+      </c>
+    </row>
+    <row r="46" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A46" s="2" t="s">
         <v>63</v>
       </c>
@@ -2059,8 +2328,14 @@
       <c r="H46" s="1">
         <v>0.29411764705882354</v>
       </c>
-    </row>
-    <row r="47" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="I46" s="3">
+        <v>48.5981308</v>
+      </c>
+      <c r="J46">
+        <v>0.117647059</v>
+      </c>
+    </row>
+    <row r="47" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A47" s="2" t="s">
         <v>64</v>
       </c>
@@ -2085,8 +2360,14 @@
       <c r="H47" s="1">
         <v>0.21554770318021199</v>
       </c>
-    </row>
-    <row r="48" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="I47" s="3">
+        <v>42.857142899999999</v>
+      </c>
+      <c r="J47">
+        <v>0.36042402800000001</v>
+      </c>
+    </row>
+    <row r="48" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A48" s="2" t="s">
         <v>65</v>
       </c>
@@ -2111,8 +2392,14 @@
       <c r="H48" s="1">
         <v>0.26147959183673469</v>
       </c>
-    </row>
-    <row r="49" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="I48" s="3">
+        <v>41.509433999999999</v>
+      </c>
+      <c r="J48">
+        <v>0.16709183699999999</v>
+      </c>
+    </row>
+    <row r="49" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A49" s="2" t="s">
         <v>66</v>
       </c>
@@ -2137,8 +2424,14 @@
       <c r="H49" s="1">
         <v>0.32035928143712578</v>
       </c>
-    </row>
-    <row r="50" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="I49" s="3">
+        <v>46.846846800000002</v>
+      </c>
+      <c r="J49">
+        <v>0.14371257500000001</v>
+      </c>
+    </row>
+    <row r="50" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A50" s="2" t="s">
         <v>67</v>
       </c>
@@ -2163,8 +2456,14 @@
       <c r="H50" s="1">
         <v>0.33521923620933525</v>
       </c>
-    </row>
-    <row r="51" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="I50" s="3">
+        <v>41.346153800000003</v>
+      </c>
+      <c r="J50">
+        <v>0.13437057999999999</v>
+      </c>
+    </row>
+    <row r="51" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A51" s="2" t="s">
         <v>68</v>
       </c>
@@ -2189,8 +2488,14 @@
       <c r="H51" s="1">
         <v>0.27089337175792505</v>
       </c>
-    </row>
-    <row r="52" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="I51" s="3">
+        <v>43.396226400000003</v>
+      </c>
+      <c r="J51">
+        <v>0.152737752</v>
+      </c>
+    </row>
+    <row r="52" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A52" s="2" t="s">
         <v>69</v>
       </c>
@@ -2215,8 +2520,14 @@
       <c r="H52" s="1">
         <v>0.31331168831168832</v>
       </c>
-    </row>
-    <row r="53" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="I52" s="3">
+        <v>46.902654900000002</v>
+      </c>
+      <c r="J52">
+        <v>0.211038961</v>
+      </c>
+    </row>
+    <row r="53" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A53" s="2" t="s">
         <v>70</v>
       </c>
@@ -2241,8 +2552,14 @@
       <c r="H53" s="1">
         <v>0.22052067381317</v>
       </c>
-    </row>
-    <row r="54" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="I53" s="3">
+        <v>58.407079600000003</v>
+      </c>
+      <c r="J53">
+        <v>0.17151607999999999</v>
+      </c>
+    </row>
+    <row r="54" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A54" s="2" t="s">
         <v>71</v>
       </c>
@@ -2267,8 +2584,14 @@
       <c r="H54" s="1">
         <v>0.30467571644042235</v>
       </c>
-    </row>
-    <row r="55" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="I54" s="3">
+        <v>53</v>
+      </c>
+      <c r="J54">
+        <v>0.177978884</v>
+      </c>
+    </row>
+    <row r="55" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A55" s="2" t="s">
         <v>72</v>
       </c>
@@ -2293,8 +2616,14 @@
       <c r="H55" s="1">
         <v>0.24911032028469748</v>
       </c>
-    </row>
-    <row r="56" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="I55" s="3">
+        <v>51.456310700000003</v>
+      </c>
+      <c r="J55">
+        <v>0.17081850500000001</v>
+      </c>
+    </row>
+    <row r="56" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A56" s="2" t="s">
         <v>73</v>
       </c>
@@ -2319,8 +2648,14 @@
       <c r="H56" s="1">
         <v>0.27160493827160498</v>
       </c>
-    </row>
-    <row r="57" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="I56" s="3">
+        <v>47.2</v>
+      </c>
+      <c r="J56">
+        <v>0.16049382700000001</v>
+      </c>
+    </row>
+    <row r="57" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A57" s="2" t="s">
         <v>74</v>
       </c>
@@ -2345,8 +2680,14 @@
       <c r="H57" s="1">
         <v>0.33075435203094777</v>
       </c>
-    </row>
-    <row r="58" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="I57" s="3">
+        <v>45.544554499999997</v>
+      </c>
+      <c r="J57">
+        <v>0.154738878</v>
+      </c>
+    </row>
+    <row r="58" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A58" s="2" t="s">
         <v>75</v>
       </c>
@@ -2371,8 +2712,14 @@
       <c r="H58" s="1">
         <v>0.12222222222222222</v>
       </c>
-    </row>
-    <row r="59" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="I58" s="3">
+        <v>42.424242399999997</v>
+      </c>
+      <c r="J58">
+        <v>0.19629629600000001</v>
+      </c>
+    </row>
+    <row r="59" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A59" s="2" t="s">
         <v>76</v>
       </c>
@@ -2397,8 +2744,14 @@
       <c r="H59" s="1">
         <v>0.27503974562798089</v>
       </c>
-    </row>
-    <row r="60" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="I59" s="3">
+        <v>44.262295100000003</v>
+      </c>
+      <c r="J59">
+        <v>0.138314785</v>
+      </c>
+    </row>
+    <row r="60" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A60" s="2" t="s">
         <v>77</v>
       </c>
@@ -2423,8 +2776,14 @@
       <c r="H60" s="1">
         <v>0.25618811881188119</v>
       </c>
-    </row>
-    <row r="61" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="I60" s="3">
+        <v>38.709677399999997</v>
+      </c>
+      <c r="J60">
+        <v>0.14603960399999999</v>
+      </c>
+    </row>
+    <row r="61" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A61" s="2" t="s">
         <v>78</v>
       </c>
@@ -2449,8 +2808,14 @@
       <c r="H61" s="1">
         <v>0.24769230769230771</v>
       </c>
-    </row>
-    <row r="62" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="I61" s="3">
+        <v>48.3333333</v>
+      </c>
+      <c r="J61">
+        <v>0.16307692300000001</v>
+      </c>
+    </row>
+    <row r="62" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A62" s="2" t="s">
         <v>79</v>
       </c>
@@ -2475,8 +2840,14 @@
       <c r="H62" s="1">
         <v>0.24172661870503598</v>
       </c>
-    </row>
-    <row r="63" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="I62" s="3">
+        <v>27.891156500000001</v>
+      </c>
+      <c r="J62">
+        <v>0.18417266199999999</v>
+      </c>
+    </row>
+    <row r="63" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A63" s="2" t="s">
         <v>80</v>
       </c>
@@ -2501,8 +2872,14 @@
       <c r="H63" s="1">
         <v>0.26242236024844723</v>
       </c>
-    </row>
-    <row r="64" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="I63" s="3">
+        <v>41.025641</v>
+      </c>
+      <c r="J63">
+        <v>0.14751552800000001</v>
+      </c>
+    </row>
+    <row r="64" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A64" s="2" t="s">
         <v>81</v>
       </c>
@@ -2527,8 +2904,14 @@
       <c r="H64" s="1">
         <v>0.27297297297297296</v>
       </c>
-    </row>
-    <row r="65" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="I64" s="3">
+        <v>42.748091600000002</v>
+      </c>
+      <c r="J64">
+        <v>0.14459459499999999</v>
+      </c>
+    </row>
+    <row r="65" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A65" s="2" t="s">
         <v>82</v>
       </c>
@@ -2553,8 +2936,14 @@
       <c r="H65" s="1">
         <v>0.22745098039215686</v>
       </c>
-    </row>
-    <row r="66" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="I65" s="3">
+        <v>36.607142899999999</v>
+      </c>
+      <c r="J65">
+        <v>0.22352941200000001</v>
+      </c>
+    </row>
+    <row r="66" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A66" s="2" t="s">
         <v>83</v>
       </c>
@@ -2579,8 +2968,14 @@
       <c r="H66" s="1">
         <v>0.34315789473684211</v>
       </c>
-    </row>
-    <row r="67" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="I66" s="3">
+        <v>32.0610687</v>
+      </c>
+      <c r="J66">
+        <v>0.13684210499999999</v>
+      </c>
+    </row>
+    <row r="67" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A67" s="2" t="s">
         <v>84</v>
       </c>
@@ -2605,8 +3000,14 @@
       <c r="H67" s="1">
         <v>0.33545647558386416</v>
       </c>
-    </row>
-    <row r="68" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="I67" s="3">
+        <v>37.6</v>
+      </c>
+      <c r="J67">
+        <v>0.159235669</v>
+      </c>
+    </row>
+    <row r="68" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A68" s="2" t="s">
         <v>85</v>
       </c>
@@ -2631,8 +3032,14 @@
       <c r="H68" s="1">
         <v>0.3</v>
       </c>
-    </row>
-    <row r="69" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="I68" s="3">
+        <v>23.8461538</v>
+      </c>
+      <c r="J68">
+        <v>0.1125</v>
+      </c>
+    </row>
+    <row r="69" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A69" s="2" t="s">
         <v>86</v>
       </c>
@@ -2657,8 +3064,14 @@
       <c r="H69" s="1">
         <v>0.34647302904564314</v>
       </c>
-    </row>
-    <row r="70" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="I69" s="3">
+        <v>31.092437</v>
+      </c>
+      <c r="J69">
+        <v>0.13485477200000001</v>
+      </c>
+    </row>
+    <row r="70" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A70" s="2" t="s">
         <v>87</v>
       </c>
@@ -2683,8 +3096,14 @@
       <c r="H70" s="1">
         <v>0.3461538461538462</v>
       </c>
-    </row>
-    <row r="71" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="I70" s="3">
+        <v>23.880597000000002</v>
+      </c>
+      <c r="J70">
+        <v>0.14230769200000001</v>
+      </c>
+    </row>
+    <row r="71" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A71" s="2" t="s">
         <v>88</v>
       </c>
@@ -2709,8 +3128,14 @@
       <c r="H71" s="1">
         <v>0.20603015075376885</v>
       </c>
-    </row>
-    <row r="72" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="I71" s="3">
+        <v>21.052631600000002</v>
+      </c>
+      <c r="J71">
+        <v>0.12060301499999999</v>
+      </c>
+    </row>
+    <row r="72" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A72" s="2" t="s">
         <v>89</v>
       </c>
@@ -2735,8 +3160,14 @@
       <c r="H72" s="1">
         <v>0.3428571428571428</v>
       </c>
-    </row>
-    <row r="73" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="I72" s="3">
+        <v>35</v>
+      </c>
+      <c r="J72">
+        <v>0.153061224</v>
+      </c>
+    </row>
+    <row r="73" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A73" s="2" t="s">
         <v>90</v>
       </c>
@@ -2761,8 +3192,14 @@
       <c r="H73" s="1">
         <v>0.32171581769436997</v>
       </c>
-    </row>
-    <row r="74" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="I73" s="3">
+        <v>49.382716000000002</v>
+      </c>
+      <c r="J73">
+        <v>0.171581769</v>
+      </c>
+    </row>
+    <row r="74" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A74" s="2" t="s">
         <v>91</v>
       </c>
@@ -2787,8 +3224,14 @@
       <c r="H74" s="1">
         <v>0.39073806078147616</v>
       </c>
-    </row>
-    <row r="75" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="I74" s="3">
+        <v>40.449438200000003</v>
+      </c>
+      <c r="J74">
+        <v>0.16063675799999999</v>
+      </c>
+    </row>
+    <row r="75" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A75" s="2" t="s">
         <v>92</v>
       </c>
@@ -2813,8 +3256,14 @@
       <c r="H75" s="1">
         <v>0.30837004405286339</v>
       </c>
-    </row>
-    <row r="76" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="I75" s="3">
+        <v>39.130434800000003</v>
+      </c>
+      <c r="J75">
+        <v>0.167400881</v>
+      </c>
+    </row>
+    <row r="76" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A76" s="2" t="s">
         <v>93</v>
       </c>
@@ -2839,8 +3288,14 @@
       <c r="H76" s="1">
         <v>0.19740259740259741</v>
       </c>
-    </row>
-    <row r="77" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="I76" s="3">
+        <v>44.230769199999997</v>
+      </c>
+      <c r="J76">
+        <v>0.18961038999999999</v>
+      </c>
+    </row>
+    <row r="77" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A77" s="2" t="s">
         <v>94</v>
       </c>
@@ -2865,8 +3320,14 @@
       <c r="H77" s="1">
         <v>0.20881670533642691</v>
       </c>
-    </row>
-    <row r="78" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="I77" s="3">
+        <v>46.551724100000001</v>
+      </c>
+      <c r="J77">
+        <v>0.16937355000000001</v>
+      </c>
+    </row>
+    <row r="78" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A78" s="2" t="s">
         <v>95</v>
       </c>
@@ -2891,8 +3352,14 @@
       <c r="H78" s="1">
         <v>0.30368763557483736</v>
       </c>
-    </row>
-    <row r="79" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="I78" s="3">
+        <v>25.471698100000001</v>
+      </c>
+      <c r="J78">
+        <v>0.15618221299999999</v>
+      </c>
+    </row>
+    <row r="79" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A79" s="2" t="s">
         <v>96</v>
       </c>
@@ -2917,8 +3384,14 @@
       <c r="H79" s="1">
         <v>0.27315541601255888</v>
       </c>
-    </row>
-    <row r="80" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="I79" s="3">
+        <v>42.7184466</v>
+      </c>
+      <c r="J79">
+        <v>0.19780219800000001</v>
+      </c>
+    </row>
+    <row r="80" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A80" s="2" t="s">
         <v>97</v>
       </c>
@@ -2943,8 +3416,14 @@
       <c r="H80" s="1">
         <v>0.31782945736434109</v>
       </c>
-    </row>
-    <row r="81" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="I80" s="3">
+        <v>41.592920399999997</v>
+      </c>
+      <c r="J80">
+        <v>0.28372092999999998</v>
+      </c>
+    </row>
+    <row r="81" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A81" s="2" t="s">
         <v>98</v>
       </c>
@@ -2969,8 +3448,14 @@
       <c r="H81" s="1">
         <v>0.30700447093889716</v>
       </c>
-    </row>
-    <row r="82" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="I81" s="3">
+        <v>41.818181799999998</v>
+      </c>
+      <c r="J81">
+        <v>0.174366617</v>
+      </c>
+    </row>
+    <row r="82" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A82" s="2" t="s">
         <v>99</v>
       </c>
@@ -2995,8 +3480,14 @@
       <c r="H82" s="1">
         <v>0.30634920634920637</v>
       </c>
-    </row>
-    <row r="83" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="I82" s="3">
+        <v>44.660194199999999</v>
+      </c>
+      <c r="J82">
+        <v>0.18412698399999999</v>
+      </c>
+    </row>
+    <row r="83" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A83" s="2" t="s">
         <v>100</v>
       </c>
@@ -3021,8 +3512,14 @@
       <c r="H83" s="1">
         <v>0.31177829099307158</v>
       </c>
-    </row>
-    <row r="84" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="I83" s="3">
+        <v>44.761904800000003</v>
+      </c>
+      <c r="J83">
+        <v>0.19630485</v>
+      </c>
+    </row>
+    <row r="84" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A84" s="2" t="s">
         <v>101</v>
       </c>
@@ -3047,8 +3544,14 @@
       <c r="H84" s="1">
         <v>0.30228758169934644</v>
       </c>
-    </row>
-    <row r="85" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="I84" s="3">
+        <v>54.545454499999998</v>
+      </c>
+      <c r="J84">
+        <v>0.16176470600000001</v>
+      </c>
+    </row>
+    <row r="85" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A85" s="2" t="s">
         <v>102</v>
       </c>
@@ -3073,8 +3576,14 @@
       <c r="H85" s="1">
         <v>0.16666666666666669</v>
       </c>
-    </row>
-    <row r="86" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="I85" s="3">
+        <v>47.663551400000003</v>
+      </c>
+      <c r="J85">
+        <v>8.4848485000000001E-2</v>
+      </c>
+    </row>
+    <row r="86" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A86" s="2" t="s">
         <v>103</v>
       </c>
@@ -3099,8 +3608,14 @@
       <c r="H86" s="1">
         <v>0.27707454289732775</v>
       </c>
-    </row>
-    <row r="87" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="I86" s="3">
+        <v>0</v>
+      </c>
+      <c r="J86">
+        <v>0.136427567</v>
+      </c>
+    </row>
+    <row r="87" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A87" s="2" t="s">
         <v>104</v>
       </c>
@@ -3125,8 +3640,14 @@
       <c r="H87" s="1">
         <v>0.20473773265651438</v>
       </c>
-    </row>
-    <row r="88" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="I87" s="3">
+        <v>20.689655200000001</v>
+      </c>
+      <c r="J87">
+        <v>0.14043993199999999</v>
+      </c>
+    </row>
+    <row r="88" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A88" s="2" t="s">
         <v>105</v>
       </c>
@@ -3151,8 +3672,14 @@
       <c r="H88" s="1">
         <v>0.14974182444061962</v>
       </c>
-    </row>
-    <row r="89" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="I88" s="3">
+        <v>0</v>
+      </c>
+      <c r="J88">
+        <v>0.22030981099999999</v>
+      </c>
+    </row>
+    <row r="89" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A89" s="2" t="s">
         <v>106</v>
       </c>
@@ -3177,8 +3704,14 @@
       <c r="H89" s="1">
         <v>0.27768860353130015</v>
       </c>
-    </row>
-    <row r="90" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="I89" s="3">
+        <v>22.3300971</v>
+      </c>
+      <c r="J89">
+        <v>0.125200642</v>
+      </c>
+    </row>
+    <row r="90" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A90" s="2" t="s">
         <v>107</v>
       </c>
@@ -3203,8 +3736,14 @@
       <c r="H90" s="1">
         <v>0.27288135593220342</v>
       </c>
-    </row>
-    <row r="91" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="I90" s="3">
+        <v>0</v>
+      </c>
+      <c r="J90">
+        <v>0.138983051</v>
+      </c>
+    </row>
+    <row r="91" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A91" s="2" t="s">
         <v>108</v>
       </c>
@@ -3229,8 +3768,14 @@
       <c r="H91" s="1">
         <v>0.25094339622641509</v>
       </c>
-    </row>
-    <row r="92" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="I91" s="3">
+        <v>29.914529900000002</v>
+      </c>
+      <c r="J91">
+        <v>0.156603774</v>
+      </c>
+    </row>
+    <row r="92" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A92" s="2" t="s">
         <v>109</v>
       </c>
@@ -3255,8 +3800,14 @@
       <c r="H92" s="1">
         <v>0.11881188118811881</v>
       </c>
-    </row>
-    <row r="93" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="I92" s="3">
+        <v>17.117117100000002</v>
+      </c>
+      <c r="J92">
+        <v>0.20792079199999999</v>
+      </c>
+    </row>
+    <row r="93" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A93" s="2" t="s">
         <v>110</v>
       </c>
@@ -3281,8 +3832,14 @@
       <c r="H93" s="1">
         <v>0.2395604395604396</v>
       </c>
-    </row>
-    <row r="94" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="I93" s="3">
+        <v>16.8141593</v>
+      </c>
+      <c r="J93">
+        <v>0.24835164800000001</v>
+      </c>
+    </row>
+    <row r="94" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A94" s="2" t="s">
         <v>111</v>
       </c>
@@ -3307,8 +3864,14 @@
       <c r="H94" s="1">
         <v>0.20285714285714285</v>
       </c>
-    </row>
-    <row r="95" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="I94" s="3">
+        <v>42.307692299999999</v>
+      </c>
+      <c r="J94">
+        <v>0.245714286</v>
+      </c>
+    </row>
+    <row r="95" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A95" s="2" t="s">
         <v>112</v>
       </c>
@@ -3333,8 +3896,14 @@
       <c r="H95" s="1">
         <v>0.16338028169014082</v>
       </c>
-    </row>
-    <row r="96" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="I95" s="3">
+        <v>41.176470600000002</v>
+      </c>
+      <c r="J95">
+        <v>0.316901408</v>
+      </c>
+    </row>
+    <row r="96" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A96" s="2" t="s">
         <v>113</v>
       </c>
@@ -3359,8 +3928,14 @@
       <c r="H96" s="1">
         <v>0.18498168498168499</v>
       </c>
-    </row>
-    <row r="97" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="I96" s="3">
+        <v>28.813559300000001</v>
+      </c>
+      <c r="J96">
+        <v>0.355311355</v>
+      </c>
+    </row>
+    <row r="97" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A97" s="2" t="s">
         <v>114</v>
       </c>
@@ -3385,8 +3960,14 @@
       <c r="H97" s="1">
         <v>0.17508417508417509</v>
       </c>
-    </row>
-    <row r="98" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="I97" s="3">
+        <v>33.076923100000002</v>
+      </c>
+      <c r="J97">
+        <v>0.42592592600000001</v>
+      </c>
+    </row>
+    <row r="98" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A98" s="2" t="s">
         <v>115</v>
       </c>
@@ -3411,8 +3992,14 @@
       <c r="H98" s="1">
         <v>0.27551020408163263</v>
       </c>
-    </row>
-    <row r="99" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="I98" s="3">
+        <v>45.192307700000001</v>
+      </c>
+      <c r="J98">
+        <v>0.26326530599999998</v>
+      </c>
+    </row>
+    <row r="99" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A99" s="2" t="s">
         <v>116</v>
       </c>
@@ -3437,11 +4024,11 @@
       <c r="H99" s="1">
         <v>0.1461794019933555</v>
       </c>
-    </row>
-    <row r="100" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="G100" s="1">
-        <f>MAX(G2:G99)</f>
-        <v>2.7</v>
+      <c r="I99" s="3">
+        <v>38.613861399999998</v>
+      </c>
+      <c r="J99">
+        <v>0.27906976700000002</v>
       </c>
     </row>
   </sheetData>

</xml_diff>